<commit_message>
Add Q3 industry benchmarks from Strategic Graphs.
Record the seven-firm comparison for capacity, market share, marketing inputs, HR,
and scorecard, which confirms operating capacity was scheduled at 8/day against 24
owned. Two corrections follow: under-scheduling also raised labor cost per unit from
130 to 205, and productivity is mid-pack rather than lagging, so the 85 percent
planning assumption was the actual error.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -31,6 +31,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Financials" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Unit_Economics" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4_Planner" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Industry_Graphs" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -43,7 +44,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -229,6 +230,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
     </font>
   </fonts>
   <fills count="33">
@@ -602,7 +607,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="169">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -834,6 +839,10 @@
     <xf numFmtId="0" fontId="28" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18112,8 +18121,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" style="146" min="1" max="1"/>
+    <col width="16" customWidth="1" style="146" min="2" max="2"/>
+    <col width="26" customWidth="1" style="146" min="3" max="3"/>
+    <col width="24" customWidth="1" style="146" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="165" t="inlineStr">
@@ -18123,9 +18138,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Rule: OC/day = forecast demand / 65 * (1 + (1 - productivity)). Never schedule below forecast again.</t>
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Rule: OC/day = forecast demand / 65 * (1 + (1 - productivity)). Never schedule below forecast again. Q3 proof: OC 8/day vs 24 owned -&gt; 204 stock-outs AND labor cost/unit up $130-&gt;$205.</t>
         </is>
       </c>
     </row>
@@ -18187,7 +18202,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>YELLOW — more people, Rio live, ads maturing</t>
+          <t>Q3 demand growth was +235% (highest in industry) on 2 stores; 1.25x is conservative</t>
         </is>
       </c>
     </row>
@@ -18214,11 +18229,11 @@
         </is>
       </c>
       <c r="B8" s="168" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>YELLOW — raise with better pay</t>
+          <t>Graph-checked: industry runs 68-73%. Assume 74% WITH a pay raise. Never plan on 85%.</t>
         </is>
       </c>
     </row>
@@ -18466,6 +18481,2007 @@
       <c r="D25" t="inlineStr">
         <is>
           <t>Lowest in industry because volume is lowest</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="166" t="inlineStr">
+        <is>
+          <t>INDUSTRY BENCHMARKS FOR Q4 (from Strategic Graphs)</t>
+        </is>
+      </c>
+      <c r="B28" s="166" t="inlineStr">
+        <is>
+          <t>WeBike Q3</t>
+        </is>
+      </c>
+      <c r="C28" s="166" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="D28" s="166" t="inlineStr">
+        <is>
+          <t>Q4 target</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Scheduled operating capacity [units/day]</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>8</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>14 - 30</t>
+        </is>
+      </c>
+      <c r="D29" s="168" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Fixed capacity [units/day]</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>24</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16 - 32</t>
+        </is>
+      </c>
+      <c r="D30" s="168" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Overtime capacity [units/day]</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>0 - 7</t>
+        </is>
+      </c>
+      <c r="D31" s="168" t="inlineStr">
+        <is>
+          <t>0 - 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Average COGS per unit [$]</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>620</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>BB LLC lowest</t>
+        </is>
+      </c>
+      <c r="D32" s="168" t="inlineStr">
+        <is>
+          <t>&lt; 550</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Average labor cost per unit [$]</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>205</v>
+      </c>
+      <c r="D33" s="168" t="inlineStr">
+        <is>
+          <t>&lt; 150</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sales compensation [$]</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>24425</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>22,000 - 27,000</t>
+        </is>
+      </c>
+      <c r="D34" s="168" t="n">
+        <v>26500</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Production compensation [$]</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>20757</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>20,500 - 23,500</t>
+        </is>
+      </c>
+      <c r="D35" s="168" t="n">
+        <v>22500</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Demand per sales person</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>45</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>60 typical / 72 best</t>
+        </is>
+      </c>
+      <c r="D36" s="168" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Store + web center spend [$]</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>121000</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>up to 360,000</t>
+        </is>
+      </c>
+      <c r="D37" s="168" t="inlineStr">
+        <is>
+          <t>raise — open city #3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Organic SEM clicks</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>150</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>440 best</t>
+        </is>
+      </c>
+      <c r="D38" s="168" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Number of stores</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2 (all but Bike Bros)</t>
+        </is>
+      </c>
+      <c r="D39" s="168" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="165" t="inlineStr">
+        <is>
+          <t>UNIT-COST UPSIDE — why right-sizing OC pays twice</t>
+        </is>
+      </c>
+      <c r="B42" s="165" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Q3 COGS per unit</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Target COGS per unit at ~15/day scale</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Saving per unit</t>
+        </is>
+      </c>
+      <c r="B45">
+        <f>B43-B44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Q4 forecast units</t>
+        </is>
+      </c>
+      <c r="B46">
+        <f>B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>COGS saving on forecast volume</t>
+        </is>
+      </c>
+      <c r="B47">
+        <f>B45*B46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>+ Gross margin recovered from ending stock-outs</t>
+        </is>
+      </c>
+      <c r="B48">
+        <f>Q3_Unit_Economics!I6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <f> Combined Q4 swing vs Q3 behaviour</f>
+        <v/>
+      </c>
+      <c r="B49" s="159">
+        <f>B47+B48</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F107"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" style="146" min="1" max="1"/>
+    <col width="16" customWidth="1" style="146" min="2" max="2"/>
+    <col width="16" customWidth="1" style="146" min="3" max="3"/>
+    <col width="22" customWidth="1" style="146" min="4" max="4"/>
+    <col width="22" customWidth="1" style="146" min="5" max="5"/>
+    <col width="60" customWidth="1" style="146" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Q3 Strategic Graphs — industry comparison (WeBike vs 6 rivals)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Source: Strategic Graphs &gt; Workspace, Quarter 4 view (shows Q0-Q3 actuals). Chart-read values are approximate; numeric report values live in Q3_BSC / Q3_Market / Q3_Financials.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>MANUFACTURING — capacity (units/day)</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>WeBike fixed capacity</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>24</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3 printers; tied 2nd highest in industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>WeBike SCHEDULED operating capacity</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C6" s="167" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CONFIRMS the back-solve: we cut OC by 60%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>WeBike overtime capacity</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ran OT on top of a tiny base</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SpaceBikes operating capacity</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>20</v>
+      </c>
+      <c r="C8" t="n">
+        <v>30</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>leader — expanded fixed capacity to 32</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MILC Bikes operating capacity</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Bike Bros operating capacity</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LiteCycle operating capacity</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>8</v>
+      </c>
+      <c r="C11" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>BB LLC operating capacity</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" t="n">
+        <v>15</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>+ ~7 overtime — highest OT in industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Spoke'd Up operating capacity</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WeBike RANK on operating capacity</t>
+        </is>
+      </c>
+      <c r="C14" s="167" t="inlineStr">
+        <is>
+          <t>LAST (7 of 7)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Only firm that REDUCED operating capacity in Q3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="166" t="inlineStr">
+        <is>
+          <t>MANUFACTURING — WeBike unit costs</t>
+        </is>
+      </c>
+      <c r="B16" s="166" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C16" s="166" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D16" s="166" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Capacity utilization [%]</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>16</v>
+      </c>
+      <c r="C17" t="n">
+        <v>73</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Q2 = idle plant; Q3 = tight plant, but tiny plant</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Average labor cost per unit [$]</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>130</v>
+      </c>
+      <c r="C18" s="167" t="n">
+        <v>205</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ROSE 58% — small OC + overtime is expensive per unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Average cost of goods sold per unit [$]</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>520</v>
+      </c>
+      <c r="C19" s="167" t="n">
+        <v>620</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ROSE ~19% despite selling 4x the units</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Production cost [$]</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>100928</v>
+      </c>
+      <c r="C20" t="n">
+        <v>272340</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Stock-outs [units]</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="n">
+        <v>204</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>the whipsaw</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Excess capacity cost [$]</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>148652</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>the whipsaw, other direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Lesson</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Under-scheduling cost us BOTH revenue AND margin. Volume normally lowers unit cost; we broke that by running a sub-scale OC with overtime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="166" t="inlineStr">
+        <is>
+          <t>MARKET — segment size (units)</t>
+        </is>
+      </c>
+      <c r="B25" s="166" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="C25" s="166" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="D25" s="166" t="inlineStr">
+        <is>
+          <t>Growth</t>
+        </is>
+      </c>
+      <c r="E25" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C26" t="n">
+        <v>2878</v>
+      </c>
+      <c r="D26">
+        <f>C25/B25-1</f>
+        <v/>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LARGEST and fastest growing; all 7 firms compete</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1100</v>
+      </c>
+      <c r="C27" t="n">
+        <v>2060</v>
+      </c>
+      <c r="D27">
+        <f>C26/B26-1</f>
+        <v/>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>we do not compete</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1621</v>
+      </c>
+      <c r="D28">
+        <f>C27/B27-1</f>
+        <v/>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>SMALLEST and slowest; our primary; only 4 firms</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Total market</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3700</v>
+      </c>
+      <c r="C29" t="n">
+        <v>6559</v>
+      </c>
+      <c r="D29">
+        <f>C28/B28-1</f>
+        <v/>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Strategic tension: our least-crowded segment is also the smallest and slowest-growing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="166" t="inlineStr">
+        <is>
+          <t>MARKET — searches (web interest, Q3)</t>
+        </is>
+      </c>
+      <c r="B31" s="166" t="inlineStr">
+        <is>
+          <t>Approx</t>
+        </is>
+      </c>
+      <c r="C31" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1350</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>highest search volume — segment we ignore</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1030</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>900</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>large demand but lowest search volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="166" t="inlineStr">
+        <is>
+          <t>MARKET — Q3 share by segment [%]</t>
+        </is>
+      </c>
+      <c r="B36" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="C36" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="D36" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="E36" s="166" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="F36" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="C37" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="D37" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="E37" t="n">
+        <v>23</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>LEADER — all 3 segments, dominates Mountain</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="E38" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>#2 — Rec + Speed only, no Mountain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="E39" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="C40" t="n">
+        <v>21</v>
+      </c>
+      <c r="D40" t="n">
+        <v>19</v>
+      </c>
+      <c r="E40" t="n">
+        <v>15</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>our closest Mountain rival</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="E41" t="n">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="C42" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E42" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>#2 Mountain, 6th Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="C43" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="D43" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="E43" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>FALLING in every segment (Mtn 19-&gt;11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="166" t="inlineStr">
+        <is>
+          <t>MARKET — demand productivity per head (Q3, approx)</t>
+        </is>
+      </c>
+      <c r="B45" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C45" s="166" t="inlineStr">
+        <is>
+          <t>Industry best</t>
+        </is>
+      </c>
+      <c r="D45" s="166" t="inlineStr">
+        <is>
+          <t>Industry typical</t>
+        </is>
+      </c>
+      <c r="E45" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Demand per sales person</t>
+        </is>
+      </c>
+      <c r="B46" s="167" t="n">
+        <v>45</v>
+      </c>
+      <c r="C46" t="n">
+        <v>72</v>
+      </c>
+      <c r="D46" t="n">
+        <v>60</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LAST — every rival gets more demand per head</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Demand per store sales person</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>46</v>
+      </c>
+      <c r="C47" t="n">
+        <v>88</v>
+      </c>
+      <c r="D47" t="n">
+        <v>70</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>BB LLC ~88; our stores under-produce</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Demand per web sales center person</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>42</v>
+      </c>
+      <c r="C48" t="n">
+        <v>95</v>
+      </c>
+      <c r="D48" t="n">
+        <v>75</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>we CUT web staff in Q3 — wrong lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Total sales people</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>14</v>
+      </c>
+      <c r="C49" t="n">
+        <v>21</v>
+      </c>
+      <c r="D49" t="n">
+        <v>14</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>headcount is at parity; output per head is not</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="166" t="inlineStr">
+        <is>
+          <t>MARKET — demand vs units sold (the leakage)</t>
+        </is>
+      </c>
+      <c r="B51" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C51" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>WeBike share of total DEMAND [%]</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>what we created</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>WeBike share of UNITS SOLD [%]</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>what we captured</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Leakage [pct points]</t>
+        </is>
+      </c>
+      <c r="B54">
+        <f>B48-B49</f>
+        <v/>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>pure stock-out loss, visible in the graphs</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Q3 demand growth rate [%]</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>235</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>highest in industry — demand generation is NOT our problem</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="166" t="inlineStr">
+        <is>
+          <t>MARKETING INPUTS (Q3, approx)</t>
+        </is>
+      </c>
+      <c r="B57" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C57" s="166" t="inlineStr">
+        <is>
+          <t>Industry high</t>
+        </is>
+      </c>
+      <c r="D57" s="166" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="E57" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Advertising expenses [$]</t>
+        </is>
+      </c>
+      <c r="B58" s="159" t="n">
+        <v>119165</v>
+      </c>
+      <c r="C58" t="n">
+        <v>145000</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>spend is competitive</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Total regional ads [count]</t>
+        </is>
+      </c>
+      <c r="B59" s="159" t="n">
+        <v>19</v>
+      </c>
+      <c r="C59" t="n">
+        <v>24</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>2nd</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ad VOLUME is a strength</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Organic SEM clicks</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>150</v>
+      </c>
+      <c r="C60" t="n">
+        <v>440</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>6th</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>weak; BB LLC 440, SpaceBikes 400</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Organic SEM expenses [$]</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C61" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Bike Bros spends 5k for 200 clicks — poor ROI benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Average price [$]</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1400</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1480</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>BB LLC prices HIGHER and still leads share</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Number of stores</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>tied</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>everyone but Bike Bros has 2 -&gt; city #3 is a differentiator</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Number of web sales centers</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>tied</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Store + web center expenses [$]</t>
+        </is>
+      </c>
+      <c r="B65" s="167" t="n">
+        <v>121000</v>
+      </c>
+      <c r="C65" t="n">
+        <v>360000</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>lowest</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>we UNDER-invest in channel</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="166" t="inlineStr">
+        <is>
+          <t>HUMAN RESOURCES (Q3, approx) — CORRECTS earlier read</t>
+        </is>
+      </c>
+      <c r="B67" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C67" s="166" t="inlineStr">
+        <is>
+          <t>Industry range</t>
+        </is>
+      </c>
+      <c r="D67" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Production worker compensation [$]</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>20757</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>20,500 - 23,500</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>low end, not an outlier</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Sales force compensation [$]</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>24425</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>22,000 - 27,000</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>middle; MILC ~27k, BB LLC ~26.5k highest</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Production worker productivity [%]</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>72</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>68 - 73</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>MID-PACK, not behind</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Sales force productivity [%]</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>70</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>70 - 75</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>MID-PACK; BB LLC ~75 best</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Comp satisfaction</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>68</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>65 - 72</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="168" t="inlineStr">
+        <is>
+          <t>CORRECTION</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>The whole industry runs ~70%. Our 85% projection was never realistic. The error was PLANNING CAPACITY on 85%, not being badly underpaid. Pay raises buy a few points, not 15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="166" t="inlineStr">
+        <is>
+          <t>BALANCED SCORECARD — Q3 by firm (approx from graph)</t>
+        </is>
+      </c>
+      <c r="B75" s="166" t="inlineStr">
+        <is>
+          <t>Total Perf</t>
+        </is>
+      </c>
+      <c r="C75" s="166" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="D75" s="166" t="inlineStr">
+        <is>
+          <t>Market</t>
+        </is>
+      </c>
+      <c r="E75" s="166" t="inlineStr">
+        <is>
+          <t>Asset Mgmt</t>
+        </is>
+      </c>
+      <c r="F75" s="166" t="inlineStr">
+        <is>
+          <t>Wealth</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>22</v>
+      </c>
+      <c r="C76" t="n">
+        <v>37.7</v>
+      </c>
+      <c r="D76" t="n">
+        <v>0.345</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>11</v>
+      </c>
+      <c r="C77" t="n">
+        <v>34</v>
+      </c>
+      <c r="D77" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E77" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="C78" t="n">
+        <v>15</v>
+      </c>
+      <c r="D78" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="E78" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C79" t="n">
+        <v>14</v>
+      </c>
+      <c r="D79" t="n">
+        <v>0.08500000000000001</v>
+      </c>
+      <c r="E79" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="D80" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="E80" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" t="n">
+        <v>6</v>
+      </c>
+      <c r="D81" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E81" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="167" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B82" s="167" t="n">
+        <v>0.411</v>
+      </c>
+      <c r="C82" s="167" t="n">
+        <v>5.319</v>
+      </c>
+      <c r="D82" s="167" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="E82" s="167" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="F82" s="167" t="n">
+        <v>0.668</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="166" t="inlineStr">
+        <is>
+          <t>CUMULATIVE BSC (approx)</t>
+        </is>
+      </c>
+      <c r="B84" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C84" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>cumulative leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>closing fast — Q3 single-quarter leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0.033</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Q2 Manufacturing Productivity of 0.20 still poisons the cumulative product</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="166" t="inlineStr">
+        <is>
+          <t>RIVAL PROFILES — what to copy and what to avoid</t>
+        </is>
+      </c>
+      <c r="B93" s="166" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>BB LLC (leader)</t>
+        </is>
+      </c>
+      <c r="B94" s="170" t="inlineStr">
+        <is>
+          <t>All 3 segments. Highest price (~$1,480) AND highest share. Most regional ads (24). Asset Mgmt 0.920 — best capital efficiency. Runs heavy overtime (~7) on modest fixed capacity: buys flexibility instead of printers. 21 sales people, ~88 demand per store rep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>SpaceBikes (cumulative leader)</t>
+        </is>
+      </c>
+      <c r="B95" s="170" t="inlineStr">
+        <is>
+          <t>Skips Mountain entirely; owns Recreation (34.5%) + Speed (20.4%). Expanded fixed capacity to 32/day — the only firm that out-built us. Highest ad spend (~$145k). Wealth 0.95.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B96" s="170" t="inlineStr">
+        <is>
+          <t>Our Mountain rival at 21.0%, plus 19.0% of Speed. Organic SEM clicks COLLAPSED 400-&gt;180.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Bike Bros (cautionary tale)</t>
+        </is>
+      </c>
+      <c r="B97" s="170" t="inlineStr">
+        <is>
+          <t>1 store, 0 web sales centers, 7 sales people. Share falling in all three segments (Mountain 19-&gt;11). Under-channeling is fatal — this is the risk of our 'cut web spend' instinct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>MILC / Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B98" s="170" t="inlineStr">
+        <is>
+          <t>Mid-pack. Spoke'd Up has the highest market growth but lowest Marketing Effectiveness (0.66).</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="166" t="inlineStr">
+        <is>
+          <t>Q4 IMPLICATIONS FROM THE GRAPHS</t>
+        </is>
+      </c>
+      <c r="B100" s="166" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1. Operating capacity</t>
+        </is>
+      </c>
+      <c r="B101" s="170" t="inlineStr">
+        <is>
+          <t>We were LAST at 8/day while owning 24. Schedule to forecast (~15/day). This is confirmed by the Operating Capacity chart, not just inferred.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2. Unit cost</t>
+        </is>
+      </c>
+      <c r="B102" s="170" t="inlineStr">
+        <is>
+          <t>Labor cost/unit rose $130-&gt;$205 and COGS/unit $520-&gt;$620 because OC was sub-scale. Right-sizing OC cuts unit cost AND ends stock-outs — one decision, two wins.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>3. Do NOT cut channel</t>
+        </is>
+      </c>
+      <c r="B103" s="170" t="inlineStr">
+        <is>
+          <t>Store+web spend is the LOWEST in industry and demand per head is LAST. Bike Bros shows where that path ends. Open city #3 and re-staff web.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>4. Pay expectations</t>
+        </is>
+      </c>
+      <c r="B104" s="170" t="inlineStr">
+        <is>
+          <t>Industry productivity is ~70% across the board. Raise pay to upper-quartile (sales ~$26-27k, production ~$22-23k) but PLAN on ~73-75%, not 85%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>5. Segment strategy</t>
+        </is>
+      </c>
+      <c r="B105" s="170" t="inlineStr">
+        <is>
+          <t>Mountain is the smallest, slowest segment (1,621) and BB LLC holds 46%. Speed is 2,878 and growing. Recreation has the most searches (1,350) and we hold 2.6%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>6. Price</t>
+        </is>
+      </c>
+      <c r="B106" s="170" t="inlineStr">
+        <is>
+          <t>BB LLC charges MORE than us and leads. Our ~$1,400 average is not the constraint — supply is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>7. Advertising</t>
+        </is>
+      </c>
+      <c r="B107" s="170" t="inlineStr">
+        <is>
+          <t>Ad count 2nd, spend 3rd, Marketing Effectiveness at par. Marketing is NOT the problem. Weakest marketing input is organic SEM clicks (150 vs 440).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record Q3 brand judgment for all 20 industry brands.
Hike Bike ties the industry ceiling in Mountain at 73, and BB LLC holds an identical
design with 2.1x our share, so the Mountain gap is supply and coverage rather than
product. Swift Bike is the second-weakest Speed brand at 72 against a 77 ceiling,
which argues for redesign rather than abandoning the segment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -32,6 +32,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Unit_Economics" sheetId="24" state="visible" r:id="rId24"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4_Planner" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Industry_Graphs" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Brand_Judgment" sheetId="27" state="visible" r:id="rId27"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -236,7 +237,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -402,6 +403,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -607,7 +613,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="171">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -841,6 +847,12 @@
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -20490,6 +20502,1547 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H91"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" style="146" min="1" max="1"/>
+    <col width="18" customWidth="1" style="146" min="2" max="2"/>
+    <col width="16" customWidth="1" style="146" min="3" max="3"/>
+    <col width="20" customWidth="1" style="146" min="4" max="4"/>
+    <col width="70" customWidth="1" style="146" min="5" max="5"/>
+    <col width="14" customWidth="1" style="146" min="6" max="6"/>
+    <col width="12" customWidth="1" style="146" min="7" max="7"/>
+    <col width="20" customWidth="1" style="146" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Brand Judgment — World Market, Q3 actual (all 20 industry brands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Score = segment appeal of the brand DESIGN (1 = no appeal). Exact figures from the sim report. A score of 1 means the brand is irrelevant to that segment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Best score</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>Gap to segment best</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>12</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>77</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>77</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>56</v>
+      </c>
+      <c r="D6" t="n">
+        <v>73</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>73</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mach 0.6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>61</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>61</v>
+      </c>
+      <c r="H7" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TERRAMean</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>59</v>
+      </c>
+      <c r="D8" t="n">
+        <v>72</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>72</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MountainCruise1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>76</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>76</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>12</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>77</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>77</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>74</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>74</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>58</v>
+      </c>
+      <c r="D12" t="n">
+        <v>70</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>70</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B13" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C13" s="171" t="n">
+        <v>56</v>
+      </c>
+      <c r="D13" s="171" t="n">
+        <v>73</v>
+      </c>
+      <c r="E13" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="171" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G13" s="171" t="n">
+        <v>73</v>
+      </c>
+      <c r="H13" s="171" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B14" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C14" s="171" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="171" t="n">
+        <v>72</v>
+      </c>
+      <c r="F14" s="171" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G14" s="171" t="n">
+        <v>72</v>
+      </c>
+      <c r="H14" s="171" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>56</v>
+      </c>
+      <c r="D15" t="n">
+        <v>73</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>73</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>74</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>74</v>
+      </c>
+      <c r="H16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>58</v>
+      </c>
+      <c r="D17" t="n">
+        <v>70</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>70</v>
+      </c>
+      <c r="H17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>9</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>76</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>76</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>73</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>73</v>
+      </c>
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>10</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>75</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>75</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>9</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="n">
+        <v>76</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>76</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>73</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>73</v>
+      </c>
+      <c r="H22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>74</v>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>74</v>
+      </c>
+      <c r="H23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>9</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>76</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>76</v>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="166" t="inlineStr">
+        <is>
+          <t>SEGMENT CEILINGS — what the best design achieves</t>
+        </is>
+      </c>
+      <c r="B26" s="166" t="inlineStr">
+        <is>
+          <t>Best score</t>
+        </is>
+      </c>
+      <c r="C26" s="166" t="inlineStr">
+        <is>
+          <t>Who holds it</t>
+        </is>
+      </c>
+      <c r="D26" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="E26" s="166" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>73</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Hike Bike (WeBike), TERRAMAX (Bike Bros), Blu Ruged Ballz (BB LLC)</t>
+        </is>
+      </c>
+      <c r="D27" s="159" t="n">
+        <v>73</v>
+      </c>
+      <c r="E27" s="159" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>77</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MACH I.I (Bike Bros), LiteSpeed Pro+ (LiteCycle)</t>
+        </is>
+      </c>
+      <c r="D28" s="167" t="n">
+        <v>72</v>
+      </c>
+      <c r="E28" s="167" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>76</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MountainCruise1 (Bike Bros)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>n/a (56 spillover)</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="172" t="inlineStr">
+        <is>
+          <t>HEADLINE — Hike Bike is tied for the BEST Mountain brand in the industry</t>
+        </is>
+      </c>
+      <c r="B32" s="172" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Hike Bike Mountain judgment</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BB LLC Blu Ruged Ballz Mountain judgment</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Our Mountain share [%]</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>22.1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>BB LLC Mountain share [%]</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>46.3</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Share ratio on an IDENTICAL brand score</t>
+        </is>
+      </c>
+      <c r="B37">
+        <f>B36/B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Conclusion</t>
+        </is>
+      </c>
+      <c r="B38" s="170" t="inlineStr">
+        <is>
+          <t>BB LLC takes 2.1x our Mountain share with a brand design scored EXACTLY the same as ours. The gap is therefore NOT product. It is supply (we stocked out 33%), sales coverage (21 sales people vs our 14, ~88 demand/store rep vs our 46) and ad volume (24 vs 19). Do not redesign Hike Bike. Feed it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="166" t="inlineStr">
+        <is>
+          <t>SPEED GAP — Swift Bike is the weakest real Speed brand</t>
+        </is>
+      </c>
+      <c r="B41" s="166" t="inlineStr">
+        <is>
+          <t>Rec</t>
+        </is>
+      </c>
+      <c r="C41" s="166" t="inlineStr">
+        <is>
+          <t>Mtn</t>
+        </is>
+      </c>
+      <c r="D41" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="E41" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MACH I.I (Bike Bros)</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>12</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>77</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>co-best Speed design</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+ (LiteCycle)</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>12</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" t="n">
+        <v>77</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>co-best Speed design</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz (BB LLC)</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>9</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>The Armstrong (SpaceBikes)</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>9</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII (MILC)</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>9</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed (Spoke'd Up)</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>10</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LiteSpeed+ (LiteCycle)</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>7</v>
+      </c>
+      <c r="C48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D48" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz (BB LLC)</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>7</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="167" t="inlineStr">
+        <is>
+          <t>Swift Bike (WeBike)</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>10</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="167" t="n">
+        <v>72</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2nd WORST — 5 points off the ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Mach 0.6 (Bike Bros)</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>9</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>61</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>only brand worse than ours</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="E52" s="170" t="inlineStr">
+        <is>
+          <t>8 of 9 rival Speed brands beat Swift Bike. The winning profile (12/1/77) is nearly identical to ours (10/1/72) - so a modest redesign should close most of the 5-point gap. Combined with our Speed AD judgment of 70, weak product + weak ad explains 7.5% share in a 2,878-unit segment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="166" t="inlineStr">
+        <is>
+          <t>DESIGN CONVERGENCE — the market has found the optimal profiles</t>
+        </is>
+      </c>
+      <c r="B55" s="166" t="inlineStr">
+        <is>
+          <t>Brands sharing it</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>56 / 73 / 1  (Mountain optimum)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TERRAMAX (Bike Bros), Hike Bike (WeBike), Blu Ruged Ballz (BB LLC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>58 / 70 / 1  (Mountain, 2nd tier)</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro (LiteCycle), Blu Tail Ballz (BB LLC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>12 / 1 / 77  (Speed optimum)</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>MACH I.I (Bike Bros), LiteSpeed Pro+ (LiteCycle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>9 / 1 / 76   (Speed, 2nd tier)</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz (BB LLC), The Armstrong (SpaceBikes), Skim MILC MKII (MILC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>7 / 1 / 74   (Speed, 3rd tier)</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>LiteSpeed+ (LiteCycle), Blu Aero Ballz (BB LLC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>73 / 1 / 1   (Recreation)</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy (Spoke'd Up), Mars Rover (SpaceBikes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="B62" s="170" t="inlineStr">
+        <is>
+          <t>Multiple firms have landed on byte-identical designs. Brand design is becoming COMMODITISED - no one can win on product alone. Nobody exceeds 73 in Mountain or 77 in Speed, so those look like hard ceilings. Differentiation must come from supply, channel, ads and price.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="166" t="inlineStr">
+        <is>
+          <t>PORTFOLIO BREADTH</t>
+        </is>
+      </c>
+      <c r="B65" s="166" t="inlineStr">
+        <is>
+          <t>Brands</t>
+        </is>
+      </c>
+      <c r="C65" s="166" t="inlineStr">
+        <is>
+          <t>Segments covered</t>
+        </is>
+      </c>
+      <c r="D65" s="166" t="inlineStr">
+        <is>
+          <t>Overall share [%]</t>
+        </is>
+      </c>
+      <c r="E65" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>5</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Rec + Mtn + Speed</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>MOST brands, LOWEST share - 1 store, 0 web centers</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>4</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Rec* + Mtn + Speed</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>23</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>leader; 2 Mtn + 2 Speed brands, Rec via spillover only</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Mtn + Speed</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="173" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Mtn + Speed</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>at parity on count</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Rec + Speed</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Rec + Speed</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>cumulative LEADER on just 2 brands - skips Mountain</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Rec + Speed</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>12.2</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="E73" s="170" t="inlineStr">
+        <is>
+          <t>Brand COUNT does not drive share: Bike Bros has 5 brands and last place; SpaceBikes has 2 and leads cumulatively. A 3rd brand is NOT our priority - filling demand for the 2 we have is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="166" t="inlineStr">
+        <is>
+          <t>RECREATION SPILLOVER — a free option we are not using</t>
+        </is>
+      </c>
+      <c r="B76" s="166" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Hike Bike appeal to Recreation buyers</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Best dedicated Recreation brand (MountainCruise1)</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Recreation segment size [units]</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2060</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Recreation searches (highest of 3 segments)</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Our Recreation share [%]</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Our Recreation demand [units, untargeted]</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="B83" s="170" t="inlineStr">
+        <is>
+          <t>Hike Bike already scores 56 with Recreation buyers and pulled 54 units we never asked for. That is real latent demand in the LARGEST-search segment. But 56 vs 76 means we cannot win Recreation on spillover - it would need a dedicated brand. Park this as a Q5 option, not a Q4 one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="166" t="inlineStr">
+        <is>
+          <t>Q4 BRAND ACTIONS</t>
+        </is>
+      </c>
+      <c r="B86" s="166" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Hike Bike (Mountain)</t>
+        </is>
+      </c>
+      <c r="B87" s="174" t="inlineStr">
+        <is>
+          <t>DO NOT REDESIGN. Tied for best in industry at 73 - already at the ceiling. Every dollar should go to supplying and selling it, not improving it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Swift Bike (Speed)</t>
+        </is>
+      </c>
+      <c r="B88" s="174" t="inlineStr">
+        <is>
+          <t>REDESIGN toward the 12/1/77 profile. We are 5 points off the ceiling and 8 of 9 rival Speed brands beat us. Also strengthen the Speed ad (judgment 70).</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Third brand</t>
+        </is>
+      </c>
+      <c r="B89" s="174" t="inlineStr">
+        <is>
+          <t>NO. Bike Bros proves brand count does not buy share. Fix supply first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="B90" s="174" t="inlineStr">
+        <is>
+          <t>DEFER. Spillover of 56 is not competitive vs 76; revisit in Q5 with a dedicated design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="B91" s="174" t="inlineStr">
+        <is>
+          <t>HOLD. Our Mountain brand matches the best design and BB LLC charges ~$1,480 - we have room at $1,365, not a reason to discount.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Reverse-engineer the brand judgment model from component teardown.
Record all 20 brands across 23 components and fit point values to the score
differences, reproducing every Mountain and Speed observation exactly. Swift Bike
carries Hike Bike's 24-speed mountain drivetrain and lacks decals, which accounts
for the full five-point gap to the Speed ceiling; Hike Bike is confirmed optimal.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -33,6 +33,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4_Planner" sheetId="25" state="visible" r:id="rId25"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Industry_Graphs" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Brand_Judgment" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Components" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Design_Model" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -613,7 +615,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -854,6 +856,18 @@
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -22043,6 +22057,2160 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="146" min="1" max="1"/>
+    <col width="26" customWidth="1" style="146" min="2" max="2"/>
+    <col width="4.5" customWidth="1" style="146" min="3" max="3"/>
+    <col width="4.5" customWidth="1" style="146" min="4" max="4"/>
+    <col width="4.5" customWidth="1" style="146" min="5" max="5"/>
+    <col width="4.5" customWidth="1" style="146" min="6" max="6"/>
+    <col width="4.5" customWidth="1" style="146" min="7" max="7"/>
+    <col width="4.5" customWidth="1" style="146" min="8" max="8"/>
+    <col width="4.5" customWidth="1" style="146" min="9" max="9"/>
+    <col width="4.5" customWidth="1" style="146" min="10" max="10"/>
+    <col width="4.5" customWidth="1" style="146" min="11" max="11"/>
+    <col width="4.5" customWidth="1" style="146" min="12" max="12"/>
+    <col width="4.5" customWidth="1" style="146" min="13" max="13"/>
+    <col width="4.5" customWidth="1" style="146" min="14" max="14"/>
+    <col width="4.5" customWidth="1" style="146" min="15" max="15"/>
+    <col width="4.5" customWidth="1" style="146" min="16" max="16"/>
+    <col width="4.5" customWidth="1" style="146" min="17" max="17"/>
+    <col width="4.5" customWidth="1" style="146" min="18" max="18"/>
+    <col width="4.5" customWidth="1" style="146" min="19" max="19"/>
+    <col width="4.5" customWidth="1" style="146" min="20" max="20"/>
+    <col width="4.5" customWidth="1" style="146" min="21" max="21"/>
+    <col width="4.5" customWidth="1" style="146" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Competitors' Brands — component teardown, Q3 actual (all 20 brands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>1 = included, blank = not included. 'Base components' and 'Standard carbon fiber' are in every brand and omitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="165" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="I4" s="166" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="J4" s="166" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="K4" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="L4" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="M4" s="166" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="N4" s="166" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="O4" s="166" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="P4" s="166" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="Q4" s="166" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="R4" s="166" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="S4" s="166" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="T4" s="166" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="U4" s="166" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="V4" s="166" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1" s="146">
+      <c r="A5" s="165" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C5" s="175" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="D5" s="175" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="E5" s="175" t="inlineStr">
+        <is>
+          <t>Mach 0.6</t>
+        </is>
+      </c>
+      <c r="F5" s="175" t="inlineStr">
+        <is>
+          <t>TERRAMean</t>
+        </is>
+      </c>
+      <c r="G5" s="175" t="inlineStr">
+        <is>
+          <t>MountainCruise1</t>
+        </is>
+      </c>
+      <c r="H5" s="175" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="I5" s="175" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="J5" s="175" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="K5" s="176" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="L5" s="176" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="M5" s="175" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="N5" s="175" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="O5" s="175" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="P5" s="175" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="Q5" s="175" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="R5" s="175" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="S5" s="175" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="T5" s="175" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="U5" s="175" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="V5" s="175" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="165" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="K6" s="173" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="L6" s="173" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="165" t="inlineStr">
+        <is>
+          <t>Judgment in target segment</t>
+        </is>
+      </c>
+      <c r="C7" s="165" t="n">
+        <v>77</v>
+      </c>
+      <c r="D7" s="165" t="n">
+        <v>73</v>
+      </c>
+      <c r="E7" s="165" t="n">
+        <v>61</v>
+      </c>
+      <c r="F7" s="165" t="n">
+        <v>72</v>
+      </c>
+      <c r="G7" s="165" t="n">
+        <v>76</v>
+      </c>
+      <c r="H7" s="165" t="n">
+        <v>77</v>
+      </c>
+      <c r="I7" s="165" t="n">
+        <v>74</v>
+      </c>
+      <c r="J7" s="165" t="n">
+        <v>70</v>
+      </c>
+      <c r="K7" s="171" t="n">
+        <v>73</v>
+      </c>
+      <c r="L7" s="171" t="n">
+        <v>72</v>
+      </c>
+      <c r="M7" s="165" t="n">
+        <v>73</v>
+      </c>
+      <c r="N7" s="165" t="n">
+        <v>74</v>
+      </c>
+      <c r="O7" s="165" t="n">
+        <v>70</v>
+      </c>
+      <c r="P7" s="165" t="n">
+        <v>76</v>
+      </c>
+      <c r="Q7" s="165" t="n">
+        <v>73</v>
+      </c>
+      <c r="R7" s="165" t="n">
+        <v>75</v>
+      </c>
+      <c r="S7" s="165" t="n">
+        <v>76</v>
+      </c>
+      <c r="T7" s="165" t="n">
+        <v>73</v>
+      </c>
+      <c r="U7" s="165" t="n">
+        <v>74</v>
+      </c>
+      <c r="V7" s="165" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="166" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Comfort (relaxed)</t>
+        </is>
+      </c>
+      <c r="G9" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T9" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U9" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Rugged (rough terrain)</t>
+        </is>
+      </c>
+      <c r="D10" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Aerodynamic (speed)</t>
+        </is>
+      </c>
+      <c r="C11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="166" t="inlineStr">
+        <is>
+          <t>Tires</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Mountain - high grip</t>
+        </is>
+      </c>
+      <c r="D13" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Hybrid - road/off-road</t>
+        </is>
+      </c>
+      <c r="G14" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U14" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Racing - fast</t>
+        </is>
+      </c>
+      <c r="C15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L15" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="N15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="P15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S15" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="166" t="inlineStr">
+        <is>
+          <t>Brakes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="T17" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="C18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U18" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V18" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Standard disc</t>
+        </is>
+      </c>
+      <c r="D19" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="166" t="inlineStr">
+        <is>
+          <t>Handlebars</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Basic straight</t>
+        </is>
+      </c>
+      <c r="D21" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M21" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Comfort straight</t>
+        </is>
+      </c>
+      <c r="G22" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T22" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U22" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Basic drop down</t>
+        </is>
+      </c>
+      <c r="C23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S23" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V23" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="166" t="inlineStr">
+        <is>
+          <t>Gears</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>7 speed (1x7)</t>
+        </is>
+      </c>
+      <c r="E25" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T25" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>14 speed (2x7)</t>
+        </is>
+      </c>
+      <c r="C26" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R26" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S26" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V26" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>24 speed (3x8)</t>
+        </is>
+      </c>
+      <c r="D27" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M27" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O27" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="166" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Polymer gel all-purpose</t>
+        </is>
+      </c>
+      <c r="D29" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Polymer gel comfort</t>
+        </is>
+      </c>
+      <c r="G30" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O30" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T30" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U30" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Polymer gel racing</t>
+        </is>
+      </c>
+      <c r="C31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L31" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S31" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V31" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="166" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Reflectors</t>
+        </is>
+      </c>
+      <c r="C33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L33" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="N33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T33" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U33" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="166" t="inlineStr">
+        <is>
+          <t>Decals</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Colorful brushstrokes</t>
+        </is>
+      </c>
+      <c r="C35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="P35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S35" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V35" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="166" t="inlineStr">
+        <is>
+          <t>Lights</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="C37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="P37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="R37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="S37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U37" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="V37" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="166" t="inlineStr">
+        <is>
+          <t>Carriers</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Plastic basket</t>
+        </is>
+      </c>
+      <c r="G39" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T39" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U39" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="166" t="inlineStr">
+        <is>
+          <t>Suspension</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Front shocks</t>
+        </is>
+      </c>
+      <c r="D41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" s="178" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="T41" s="177" t="n">
+        <v>1</v>
+      </c>
+      <c r="U41" s="177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D85"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" style="146" min="1" max="1"/>
+    <col width="30" customWidth="1" style="146" min="2" max="2"/>
+    <col width="34" customWidth="1" style="146" min="3" max="3"/>
+    <col width="10" customWidth="1" style="146" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Reverse-engineered brand judgment model (fitted to all 20 brands)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Every brand in each segment shares one base recipe; scores differ only by a few components. The point values below reproduce all 20 observed scores exactly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>SPEED — base recipe (all 10 Speed brands share this)</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Aerodynamic</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tires</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Racing - fast</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Brakes</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Handlebars</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Basic drop down</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Polymer gel racing</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carriers / Suspension</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="166" t="inlineStr">
+        <is>
+          <t>SPEED — what the variable components are worth</t>
+        </is>
+      </c>
+      <c r="B13" s="166" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="C13" s="166" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Gears 14 speed (2x7)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="C14" s="170" t="inlineStr">
+        <is>
+          <t>all 8 top Speed brands use it</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Gears 24 speed (3x8) instead</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>-3</v>
+      </c>
+      <c r="C15" s="170" t="inlineStr">
+        <is>
+          <t>Swift Bike is the ONLY Speed brand with it</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gears 7 speed (1x7) instead</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-16</v>
+      </c>
+      <c r="C16" s="170" t="inlineStr">
+        <is>
+          <t>Mach 0.6 = 61 with an otherwise full kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Decals (colorful brushstrokes)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="170" t="inlineStr">
+        <is>
+          <t>every 76-77 brand has them; every 72-75 brand lacks them</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Reflectors</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="170" t="inlineStr">
+        <is>
+          <t>MACH I.I 77 (with) vs Blu Tube 76 (without), else identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lights</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" s="170" t="inlineStr">
+        <is>
+          <t>Blu Aero 74 lacks lights; otherwise matches 75-point kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>MAXIMUM ACHIEVABLE (Speed)</t>
+        </is>
+      </c>
+      <c r="B20" s="159" t="n">
+        <v>77</v>
+      </c>
+      <c r="C20" s="170" t="inlineStr">
+        <is>
+          <t>MACH I.I and LiteSpeed Pro+ both hit it</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="166" t="inlineStr">
+        <is>
+          <t>SWIFT BIKE — exact fix to reach the industry ceiling</t>
+        </is>
+      </c>
+      <c r="B23" s="166" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="C23" s="166" t="inlineStr">
+        <is>
+          <t>Change to</t>
+        </is>
+      </c>
+      <c r="D23" s="166" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Aerodynamic</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tires</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Racing</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Brakes</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Handlebars</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Basic drop down</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Polymer gel racing</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Reflectors</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>included</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Lights</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>included</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Gears</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>24 speed (3x8)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>14 speed (2x7)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Decals</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>not included</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ADD colorful brushstrokes</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Current judgment</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Projected judgment after both changes</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>B33+SUM(D32:D33)</f>
+        <v/>
+      </c>
+      <c r="C34">
+        <f> industry ceiling (tied best)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="166" t="inlineStr">
+        <is>
+          <t>Why the gears mistake happened</t>
+        </is>
+      </c>
+      <c r="B37" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Root cause</t>
+        </is>
+      </c>
+      <c r="B38" s="170" t="inlineStr">
+        <is>
+          <t>Swift Bike inherited the 24-speed (3x8) mountain drivetrain from Hike Bike. 24-speed is OPTIMAL in Mountain (all 6 Mountain brands use it) and WRONG in Speed (all 8 leading Speed brands use 14-speed). We copied our Mountain spec into a Speed bike.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Cost side effect</t>
+        </is>
+      </c>
+      <c r="B39" s="170" t="inlineStr">
+        <is>
+          <t>14 speed (2x7) is a simpler drivetrain than 24 speed (3x8), so this change should also LOWER unit cost. Verify against the component price list before locking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="166" t="inlineStr">
+        <is>
+          <t>MOUNTAIN — base recipe (all 6 Mountain brands share this)</t>
+        </is>
+      </c>
+      <c r="B42" s="166" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Rugged</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Tires</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Mountain - high grip</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Brakes</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Standard disc</t>
+        </is>
+      </c>
+      <c r="C45" s="168" t="n"/>
+      <c r="D45" s="168" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Handlebars</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Basic straight</t>
+        </is>
+      </c>
+      <c r="C46" s="168" t="n"/>
+      <c r="D46" s="168" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Gears</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>24 speed (3x8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Suspension</t>
+        </is>
+      </c>
+      <c r="B48" s="172" t="inlineStr">
+        <is>
+          <t>Front shocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Decals</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Colorful brushstrokes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Lights / Carriers</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="166" t="inlineStr">
+        <is>
+          <t>MOUNTAIN — what the variable components are worth</t>
+        </is>
+      </c>
+      <c r="B53" s="166" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="C53" s="166" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Seat: Polymer gel ALL-PURPOSE</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>optimal</t>
+        </is>
+      </c>
+      <c r="C54" s="170" t="inlineStr">
+        <is>
+          <t>Hike Bike, TERRAMAX, Blu Ruged Ballz all = 73</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Seat: Polymer gel COMFORT instead</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>-3</v>
+      </c>
+      <c r="C55" s="170" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro and Blu Tail Ballz both = 70</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Reflectors added</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>-1</v>
+      </c>
+      <c r="C56" s="170" t="inlineStr">
+        <is>
+          <t>TERRAMean = 72; identical to Hike Bike except reflectors</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>MAXIMUM ACHIEVABLE (Mountain)</t>
+        </is>
+      </c>
+      <c r="B57" s="159" t="n">
+        <v>73</v>
+      </c>
+      <c r="C57" s="170" t="inlineStr">
+        <is>
+          <t>Hike Bike already there</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" s="167" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="166" t="inlineStr">
+        <is>
+          <t>HIKE BIKE — verified optimal, do not touch</t>
+        </is>
+      </c>
+      <c r="B60" s="166" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="B61" s="170" t="inlineStr">
+        <is>
+          <t>Polymer gel all-purpose = correct (comfort seat would cost 3 points)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Reflectors</t>
+        </is>
+      </c>
+      <c r="B62" s="170" t="inlineStr">
+        <is>
+          <t>correctly EXCLUDED (adding them costs 1 point - they are a Recreation cue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Lights</t>
+        </is>
+      </c>
+      <c r="B63" s="170" t="inlineStr">
+        <is>
+          <t>correctly excluded</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Judgment</t>
+        </is>
+      </c>
+      <c r="B64" s="170" t="inlineStr">
+        <is>
+          <t>73 of a possible 73 - nothing left to gain from redesign</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Implication</t>
+        </is>
+      </c>
+      <c r="B65" s="170" t="inlineStr">
+        <is>
+          <t>Any Q4 budget aimed at improving Hike Bike is wasted. Spend it on capacity, sales coverage and ads instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="166" t="inlineStr">
+        <is>
+          <t>RECREATION — blueprint if we ever enter (Q5 option)</t>
+        </is>
+      </c>
+      <c r="B68" s="166" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Frame</t>
+        </is>
+      </c>
+      <c r="B69" s="170" t="inlineStr">
+        <is>
+          <t>Comfort (relaxed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Tires</t>
+        </is>
+      </c>
+      <c r="B70" s="170" t="inlineStr">
+        <is>
+          <t>Hybrid - road/off-road</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Brakes</t>
+        </is>
+      </c>
+      <c r="B71" s="170" t="inlineStr">
+        <is>
+          <t>Standard disc  &lt;-- NOT precision (costs 2) and NOT standard (costs 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Handlebars</t>
+        </is>
+      </c>
+      <c r="B72" s="170" t="inlineStr">
+        <is>
+          <t>Comfort straight</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Gears</t>
+        </is>
+      </c>
+      <c r="B73" s="170" t="inlineStr">
+        <is>
+          <t>7 speed (1x7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="B74" s="170" t="inlineStr">
+        <is>
+          <t>Polymer gel comfort</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="B75" s="170" t="inlineStr">
+        <is>
+          <t>Reflectors + Decals + Lights + Plastic basket + Front shocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B76" s="170" t="inlineStr">
+        <is>
+          <t>76 = MountainCruise1 (Bike Bros), the only brand at the Recreation ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>CAUTION</t>
+        </is>
+      </c>
+      <c r="B77" s="170" t="inlineStr">
+        <is>
+          <t>Only 4 Recreation brands exist and they differ in 3 places (brakes, decals, lights), so the individual penalties are NOT uniquely identifiable. Observed constraints: precision+no-decals = 2 - precision+no-lights = 3 - standard-brakes+no-decals = 3. What IS certain: standard disc brakes are optimal, and MountainCruise1's exact recipe scores 76.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="166" t="inlineStr">
+        <is>
+          <t>CROSS-SEGMENT RULE OF THUMB</t>
+        </is>
+      </c>
+      <c r="B80" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Reflectors</t>
+        </is>
+      </c>
+      <c r="B81" s="170" t="inlineStr">
+        <is>
+          <t>+1 in Speed, -1 in Mountain, required in Recreation. Segment-dependent, not universally good.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Decals</t>
+        </is>
+      </c>
+      <c r="B82" s="170" t="inlineStr">
+        <is>
+          <t>+2 in Speed, required in Mountain and Recreation. Cheap and always worth having except where noted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Lights</t>
+        </is>
+      </c>
+      <c r="B83" s="170" t="inlineStr">
+        <is>
+          <t>+1 in Speed, excluded in Mountain, required in Recreation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Gears</t>
+        </is>
+      </c>
+      <c r="B84" s="170" t="inlineStr">
+        <is>
+          <t>The single biggest lever in Speed: 7sp = -16, 24sp = -3, 14sp = optimal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="B85" s="170" t="inlineStr">
+        <is>
+          <t>The single biggest lever in Mountain: comfort seat = -3 vs all-purpose.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Map Q3 demand by city and reframe the city #3 choice.
Store the 65 brand-by-city demand rows, which reconcile exactly to the reported
totals, and derive the competitive map. A local store swings share by roughly ten
times, Rio is uncontested and carries 58 percent of its Mountain segment, and New
York offers a larger prize than Bangalore but only if attacked through Speed.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -35,6 +35,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Brand_Judgment" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Components" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Design_Model" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_City_Demand" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_City_Strategy" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -615,7 +617,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="179">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -868,6 +870,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -24522,6 +24529,3029 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" style="146" min="1" max="1"/>
+    <col width="13" customWidth="1" style="146" min="2" max="2"/>
+    <col width="16" customWidth="1" style="146" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Detailed Brand Demand — World Market by city, Q3 actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Reconciles exactly to 6,559 total / 627 WeBike / 412 Hike Bike / 215 Swift Bike.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>39</v>
+      </c>
+      <c r="G5" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>29</v>
+      </c>
+      <c r="G6" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>13</v>
+      </c>
+      <c r="E7" t="n">
+        <v>62</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B8" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C8" s="171" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D8" s="171" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="171" t="n">
+        <v>23</v>
+      </c>
+      <c r="F8" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="171" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B9" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C9" s="171" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D9" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="171" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="171" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>19</v>
+      </c>
+      <c r="E10" t="n">
+        <v>265</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>135</v>
+      </c>
+      <c r="G11" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>22</v>
+      </c>
+      <c r="E12" t="n">
+        <v>145</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>166</v>
+      </c>
+      <c r="G13" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>237</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>175</v>
+      </c>
+      <c r="G15" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>272</v>
+      </c>
+      <c r="G16" t="n">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>302</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>68</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>52</v>
+      </c>
+      <c r="G19" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>27</v>
+      </c>
+      <c r="G20" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>20</v>
+      </c>
+      <c r="G21" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>13</v>
+      </c>
+      <c r="E22" t="n">
+        <v>46</v>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B23" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C23" s="171" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D23" s="171" t="n">
+        <v>25</v>
+      </c>
+      <c r="E23" s="171" t="n">
+        <v>166</v>
+      </c>
+      <c r="F23" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="171" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B24" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C24" s="171" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D24" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="171" t="n">
+        <v>79</v>
+      </c>
+      <c r="G24" s="171" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>6</v>
+      </c>
+      <c r="E25" t="n">
+        <v>48</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>23</v>
+      </c>
+      <c r="G26" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>7</v>
+      </c>
+      <c r="E27" t="n">
+        <v>26</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>29</v>
+      </c>
+      <c r="G28" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>21</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>11</v>
+      </c>
+      <c r="G30" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>43</v>
+      </c>
+      <c r="G31" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>77</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>70</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>37</v>
+      </c>
+      <c r="G34" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>155</v>
+      </c>
+      <c r="G35" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>6</v>
+      </c>
+      <c r="E36" t="n">
+        <v>92</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Mach 0.6</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>25</v>
+      </c>
+      <c r="G37" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TERRAMean</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>10</v>
+      </c>
+      <c r="E38" t="n">
+        <v>80</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>MountainCruise1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>122</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>126</v>
+      </c>
+      <c r="G40" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>93</v>
+      </c>
+      <c r="G41" t="n">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>36</v>
+      </c>
+      <c r="E42" t="n">
+        <v>110</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B43" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C43" s="171" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D43" s="171" t="n">
+        <v>24</v>
+      </c>
+      <c r="E43" s="171" t="n">
+        <v>156</v>
+      </c>
+      <c r="F43" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="171" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B44" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C44" s="171" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D44" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="171" t="n">
+        <v>115</v>
+      </c>
+      <c r="G44" s="171" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>16</v>
+      </c>
+      <c r="E45" t="n">
+        <v>137</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>110</v>
+      </c>
+      <c r="G46" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>19</v>
+      </c>
+      <c r="E47" t="n">
+        <v>75</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>136</v>
+      </c>
+      <c r="G48" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>217</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" t="n">
+        <v>163</v>
+      </c>
+      <c r="G50" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" t="n">
+        <v>223</v>
+      </c>
+      <c r="G51" t="n">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>267</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" t="n">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>275</v>
+      </c>
+      <c r="E53" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="n">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" t="n">
+        <v>197</v>
+      </c>
+      <c r="G54" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="n">
+        <v>0</v>
+      </c>
+      <c r="F55" t="n">
+        <v>123</v>
+      </c>
+      <c r="G55" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="n">
+        <v>0</v>
+      </c>
+      <c r="F56" t="n">
+        <v>91</v>
+      </c>
+      <c r="G56" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>34</v>
+      </c>
+      <c r="E57" t="n">
+        <v>122</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B58" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C58" s="171" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D58" s="171" t="n">
+        <v>2</v>
+      </c>
+      <c r="E58" s="171" t="n">
+        <v>13</v>
+      </c>
+      <c r="F58" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="171" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B59" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C59" s="171" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D59" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" s="171" t="n">
+        <v>9</v>
+      </c>
+      <c r="G59" s="171" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>5</v>
+      </c>
+      <c r="E60" t="n">
+        <v>36</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>0</v>
+      </c>
+      <c r="E61" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" t="n">
+        <v>26</v>
+      </c>
+      <c r="G61" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>5</v>
+      </c>
+      <c r="E62" t="n">
+        <v>19</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>32</v>
+      </c>
+      <c r="G63" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>17</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>13</v>
+      </c>
+      <c r="G65" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>50</v>
+      </c>
+      <c r="G66" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>64</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>58</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0</v>
+      </c>
+      <c r="F69" t="n">
+        <v>42</v>
+      </c>
+      <c r="G69" t="n">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" style="146" min="1" max="1"/>
+    <col width="30" customWidth="1" style="146" min="2" max="2"/>
+    <col width="30" customWidth="1" style="146" min="3" max="3"/>
+    <col width="16" customWidth="1" style="146" min="4" max="4"/>
+    <col width="16" customWidth="1" style="146" min="5" max="5"/>
+    <col width="16" customWidth="1" style="146" min="6" max="6"/>
+    <col width="16" customWidth="1" style="146" min="7" max="7"/>
+    <col width="16" customWidth="1" style="146" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>City-level competitive map and the City #3 decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Amsterdam + New York are 77% of the entire market. We hold 9.9% of Amsterdam and 1.9% of New York, but 34.9% of Rio - the one city where we are the only firm with a store.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>CITY SIZE &amp; OUR POSITION</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Total demand</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>% of market</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>WeBike units</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>WeBike share</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>992</v>
+      </c>
+      <c r="C5" t="n">
+        <v>650</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1343</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2985</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>0.455099862783961</v>
+      </c>
+      <c r="G5" t="n">
+        <v>295</v>
+      </c>
+      <c r="H5" s="179" t="n">
+        <v>0.09882747068676717</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>664</v>
+      </c>
+      <c r="C6" t="n">
+        <v>495</v>
+      </c>
+      <c r="D6" t="n">
+        <v>880</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2039</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>0.3108705595365147</v>
+      </c>
+      <c r="G6" t="n">
+        <v>38</v>
+      </c>
+      <c r="H6" s="179" t="n">
+        <v>0.01863658656204022</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>219</v>
+      </c>
+      <c r="C7" t="n">
+        <v>286</v>
+      </c>
+      <c r="D7" t="n">
+        <v>269</v>
+      </c>
+      <c r="E7" t="n">
+        <v>774</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>0.1180057935660924</v>
+      </c>
+      <c r="G7" t="n">
+        <v>270</v>
+      </c>
+      <c r="H7" s="161" t="n">
+        <v>0.3488372093023256</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>185</v>
+      </c>
+      <c r="C8" t="n">
+        <v>190</v>
+      </c>
+      <c r="D8" t="n">
+        <v>386</v>
+      </c>
+      <c r="E8" t="n">
+        <v>761</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>0.1160237841134319</v>
+      </c>
+      <c r="G8" t="n">
+        <v>24</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>0.03153745072273324</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2060</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1621</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2878</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6559</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>627</v>
+      </c>
+      <c r="H9" s="10" t="n">
+        <v>0.09559384052447019</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="166" t="inlineStr">
+        <is>
+          <t>SHARE BY CITY [%] — who owns what</t>
+        </is>
+      </c>
+      <c r="B12" s="166" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="C12" s="166" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="D12" s="166" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E12" s="166" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>0.1651591289782245</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>0.3688082393330064</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>0.1795865633074935</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>0.1616294349540079</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0.1641541038525963</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0.2815105443845022</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0.1550387596899225</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0.1498028909329829</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>0.1222780569514238</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>0.07013241785188817</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>0.1369509043927649</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>0.4862023653088042</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>0.1273031825795645</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <v>0.2020598332515939</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>0.041343669250646</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>0.03942181340341656</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>0.1581239530988275</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.0588523786169691</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>0.1382428940568475</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>0.1314060446780552</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B18" s="180" t="n">
+        <v>0.09882747068676717</v>
+      </c>
+      <c r="C18" s="180" t="n">
+        <v>0.01863658656204022</v>
+      </c>
+      <c r="D18" s="180" t="n">
+        <v>0.3488372093023256</v>
+      </c>
+      <c r="E18" s="180" t="n">
+        <v>0.03153745072273324</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="n">
+        <v>0.1641541038525963</v>
+      </c>
+      <c r="C19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="166" t="inlineStr">
+        <is>
+          <t>INFERRED STORE LOCATIONS (from demand concentration)</t>
+        </is>
+      </c>
+      <c r="B22" s="166" t="inlineStr">
+        <is>
+          <t>Firms with a store</t>
+        </is>
+      </c>
+      <c r="C22" s="166" t="inlineStr">
+        <is>
+          <t>City demand</t>
+        </is>
+      </c>
+      <c r="D22" s="166" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ALL SEVEN</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2985</v>
+      </c>
+      <c r="D23" s="170" t="inlineStr">
+        <is>
+          <t>Most contested city AND the largest. Nobody exceeds 16.5%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B24" s="167" t="inlineStr">
+        <is>
+          <t>BB LLC, SpaceBikes, Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2039</v>
+      </c>
+      <c r="D24" s="170" t="inlineStr">
+        <is>
+          <t>2nd largest. We have NO store -&gt; only 1.9% share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B25" s="159" t="inlineStr">
+        <is>
+          <t>WeBike ONLY</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>774</v>
+      </c>
+      <c r="D25" s="170" t="inlineStr">
+        <is>
+          <t>Uncontested by any rival store -&gt; we take 34.9%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>LiteCycle ONLY</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>761</v>
+      </c>
+      <c r="D26" s="170" t="inlineStr">
+        <is>
+          <t>Uncontested by others -&gt; LiteCycle takes 48.6%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Amsterdam only (1 store, 0 web)</t>
+        </is>
+      </c>
+      <c r="D27" s="170" t="inlineStr">
+        <is>
+          <t>Appears in NO other city. Confirms the 1-store read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="168" t="inlineStr">
+        <is>
+          <t>CAUTION</t>
+        </is>
+      </c>
+      <c r="D28" s="170" t="inlineStr">
+        <is>
+          <t>Store locations are INFERRED from demand patterns, not reported directly. MILC Bikes is Amsterdam-concentrated but its 2nd store is not identifiable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="166" t="inlineStr">
+        <is>
+          <t>THE STORE EFFECT — what a local store is worth</t>
+        </is>
+      </c>
+      <c r="B31" s="166" t="inlineStr">
+        <is>
+          <t>Share with store</t>
+        </is>
+      </c>
+      <c r="C31" s="166" t="inlineStr">
+        <is>
+          <t>Share without store</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>WeBike in Rio (only store in city)</t>
+        </is>
+      </c>
+      <c r="B32" s="161" t="n">
+        <v>0.349</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LiteCycle in Bangalore (only store in city)</t>
+        </is>
+      </c>
+      <c r="B33" s="161" t="n">
+        <v>0.486</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>WeBike in Amsterdam (store, 6 rivals)</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>0.099</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>WeBike in New York City (no store)</t>
+        </is>
+      </c>
+      <c r="C35" s="179" t="n">
+        <v>0.019</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>WeBike in Bangalore (no store)</t>
+        </is>
+      </c>
+      <c r="C36" s="179" t="n">
+        <v>0.032</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="B37" s="170" t="inlineStr">
+        <is>
+          <t>A store is worth roughly 10x the share of web-only coverage (2-3% without, 10-35% with). An UNCONTESTED store is worth 35-49%. This is the highest-leverage decision we have.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="166" t="inlineStr">
+        <is>
+          <t>OUR PRIMARY SEGMENT (Mountain) BY CITY</t>
+        </is>
+      </c>
+      <c r="B40" s="166" t="inlineStr">
+        <is>
+          <t>Segment size</t>
+        </is>
+      </c>
+      <c r="C40" s="166" t="inlineStr">
+        <is>
+          <t>WeBike units</t>
+        </is>
+      </c>
+      <c r="D40" s="166" t="inlineStr">
+        <is>
+          <t>WeBike share</t>
+        </is>
+      </c>
+      <c r="E40" s="166" t="inlineStr">
+        <is>
+          <t>Leader</t>
+        </is>
+      </c>
+      <c r="F40" s="166" t="inlineStr">
+        <is>
+          <t>Leader units</t>
+        </is>
+      </c>
+      <c r="G40" s="166" t="inlineStr">
+        <is>
+          <t>Leader share</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>650</v>
+      </c>
+      <c r="C41" t="n">
+        <v>156</v>
+      </c>
+      <c r="D41" s="10" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>156</v>
+      </c>
+      <c r="G41" s="10" t="n">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>495</v>
+      </c>
+      <c r="C42" t="n">
+        <v>23</v>
+      </c>
+      <c r="D42" s="179" t="n">
+        <v>0.04646464646464647</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>BB LLC (both brands)</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>410</v>
+      </c>
+      <c r="G42" s="10" t="n">
+        <v>0.8282828282828283</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>286</v>
+      </c>
+      <c r="C43" t="n">
+        <v>166</v>
+      </c>
+      <c r="D43" s="161" t="n">
+        <v>0.5804195804195804</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>166</v>
+      </c>
+      <c r="G43" s="10" t="n">
+        <v>0.5804195804195804</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>190</v>
+      </c>
+      <c r="C44" t="n">
+        <v>13</v>
+      </c>
+      <c r="D44" s="10" t="n">
+        <v>0.06842105263157895</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>122</v>
+      </c>
+      <c r="G44" s="10" t="n">
+        <v>0.6421052631578947</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="166" t="inlineStr">
+        <is>
+          <t>CITY #3 DECISION — New York City vs Bangalore</t>
+        </is>
+      </c>
+      <c r="B47" s="166" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="C47" s="166" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Total city demand (Q3)</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2039</v>
+      </c>
+      <c r="C48" t="n">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Share of total market</t>
+        </is>
+      </c>
+      <c r="B49" s="10">
+        <f>B48/6559</f>
+        <v/>
+      </c>
+      <c r="C49" s="10">
+        <f>C48/6559</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Rival stores already there</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Our current share (web only)</t>
+        </is>
+      </c>
+      <c r="B51" s="10" t="n">
+        <v>0.019</v>
+      </c>
+      <c r="C51" s="10" t="n">
+        <v>0.032</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Mountain segment size</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>495</v>
+      </c>
+      <c r="C52" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Mountain leader hold</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>BB LLC 82.8%</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>LiteCycle 64.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Speed segment size</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>880</v>
+      </c>
+      <c r="C54" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Recreation segment size (untapped)</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>664</v>
+      </c>
+      <c r="C55" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Units at a conservative 10% share</t>
+        </is>
+      </c>
+      <c r="B56">
+        <f>B48*0.10</f>
+        <v/>
+      </c>
+      <c r="C56">
+        <f>C48*0.10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Units at a Rio-like 25% share</t>
+        </is>
+      </c>
+      <c r="B57">
+        <f>B48*0.25</f>
+        <v/>
+      </c>
+      <c r="C57">
+        <f>C48*0.25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>VERDICT</t>
+        </is>
+      </c>
+      <c r="B58" s="181" t="inlineStr">
+        <is>
+          <t>LARGER PRIZE — 2.7x the demand. Even at a weak 10% it beats Bangalore at 25%. Fits our locked 'largest geos even if expensive' strategy.</t>
+        </is>
+      </c>
+      <c r="C58" s="170" t="inlineStr">
+        <is>
+          <t>SAFER but SMALLER — only LiteCycle to fight, yet the whole city is worth less than NYC's Speed segment alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="166" t="inlineStr">
+        <is>
+          <t>CAPACITY CHECK — can we even serve a 3rd city?</t>
+        </is>
+      </c>
+      <c r="B61" s="166" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Fixed capacity per day</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Days per quarter</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Theoretical max units</t>
+        </is>
+      </c>
+      <c r="B64">
+        <f>B62*B63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>At 74% worker productivity</t>
+        </is>
+      </c>
+      <c r="B65">
+        <f>B64*0.74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Q4 forecast demand (existing cities, after ill will)</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Headroom for a new city</t>
+        </is>
+      </c>
+      <c r="B67" s="159">
+        <f>B65-B66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="B68" s="170" t="inlineStr">
+        <is>
+          <t>We can absorb roughly 500 more units without buying a printer. A New York store at 10% (~204 units) fits comfortably. DO NOT repeat Q3 - schedule the operating capacity to match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="166" t="inlineStr">
+        <is>
+          <t>RISKS &amp; PROTECTIONS</t>
+        </is>
+      </c>
+      <c r="B71" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Rio is our crown jewel</t>
+        </is>
+      </c>
+      <c r="B72" s="174" t="inlineStr">
+        <is>
+          <t>58.0% of Rio Mountain and 34.9% of the city. Hike Bike's single best market (166 Mountain units, more than Amsterdam's 156). The Q3 stock-out damaged our strongest position - ill will bites hardest exactly where we lead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Amsterdam is the biggest miss</t>
+        </is>
+      </c>
+      <c r="B73" s="170" t="inlineStr">
+        <is>
+          <t>2,985 units = 45.5% of the market and we hold only 9.9%. Adding sales coverage here may be cheaper per unit than a new city, and no rival exceeds 16.5% - it is genuinely open.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>New York is BB LLC's fortress</t>
+        </is>
+      </c>
+      <c r="B74" s="170" t="inlineStr">
+        <is>
+          <t>They take 36.9% of the city and 82.8% of its Mountain. Attack via SPEED (880 units, no single firm dominant) and Recreation, not head-on in Mountain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Bangalore is LiteCycle's fortress</t>
+        </is>
+      </c>
+      <c r="B75" s="170" t="inlineStr">
+        <is>
+          <t>48.6% city share, 64.2% of its Mountain - the most concentrated position any firm holds in any city.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Do not spread too thin</t>
+        </is>
+      </c>
+      <c r="B76" s="170" t="inlineStr">
+        <is>
+          <t>Bike Bros ran 5 brands from 1 store and finished last. Our constraint is supply and coverage depth, not map coverage.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Q3 channel mix and cost the web cut.
Our 120 web units are the lowest of any firm operating a web centre, and web
carries half our reach into cities without a store. Matching the industry web mix
would add roughly 152 units and 90 thousand dollars of quarterly margin, which
argues for channel depth ahead of a third city.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -37,6 +37,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Design_Model" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_City_Demand" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_City_Strategy" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Channel" sheetId="32" state="visible" r:id="rId32"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -617,7 +618,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="182">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -874,6 +875,12 @@
     <xf numFmtId="164" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="28" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="28" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -27552,6 +27559,1044 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" style="146" min="1" max="1"/>
+    <col width="20" customWidth="1" style="146" min="2" max="2"/>
+    <col width="56" customWidth="1" style="146" min="3" max="3"/>
+    <col width="15" customWidth="1" style="146" min="4" max="4"/>
+    <col width="15" customWidth="1" style="146" min="5" max="5"/>
+    <col width="15" customWidth="1" style="146" min="6" max="6"/>
+    <col width="15" customWidth="1" style="146" min="7" max="7"/>
+    <col width="15" customWidth="1" style="146" min="8" max="8"/>
+    <col width="15" customWidth="1" style="146" min="9" max="9"/>
+    <col width="15" customWidth="1" style="146" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Demand Distribution by Channel — Q3 actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>We cut web staff and spend in Q3. This is the bill: 120 web units, the lowest of any firm that operates a web centre, and 19.1% web mix against an industry average of 34.9%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Store demand</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Store %</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Web demand</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Web %</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Total demand</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Stores</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>Demand / store</t>
+        </is>
+      </c>
+      <c r="I4" s="166" t="inlineStr">
+        <is>
+          <t>Web centres</t>
+        </is>
+      </c>
+      <c r="J4" s="166" t="inlineStr">
+        <is>
+          <t>Demand / web centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>938</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0.6224286662242866</v>
+      </c>
+      <c r="D5" t="n">
+        <v>569</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>0.3775713337757133</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1507</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="182" t="n">
+        <v>469</v>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="182" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>807</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>0.6217257318952234</v>
+      </c>
+      <c r="D6" t="n">
+        <v>491</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0.3782742681047766</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1298</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="182" t="n">
+        <v>403.5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="182" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>549</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.5579268292682927</v>
+      </c>
+      <c r="D7" t="n">
+        <v>435</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>0.4420731707317073</v>
+      </c>
+      <c r="F7" t="n">
+        <v>984</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="182" t="n">
+        <v>274.5</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="182" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>716</v>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>0.8384074941451991</v>
+      </c>
+      <c r="D8" t="n">
+        <v>138</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>0.1615925058548009</v>
+      </c>
+      <c r="F8" t="n">
+        <v>854</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="182" t="n">
+        <v>358</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="182" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>364</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>0.4555694618272841</v>
+      </c>
+      <c r="D9" t="n">
+        <v>435</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>0.5444305381727159</v>
+      </c>
+      <c r="F9" t="n">
+        <v>799</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="182" t="n">
+        <v>364</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="182" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B10" s="171" t="n">
+        <v>507</v>
+      </c>
+      <c r="C10" s="183" t="n">
+        <v>0.8086124401913876</v>
+      </c>
+      <c r="D10" s="171" t="n">
+        <v>120</v>
+      </c>
+      <c r="E10" s="183" t="n">
+        <v>0.1913875598086124</v>
+      </c>
+      <c r="F10" s="171" t="n">
+        <v>627</v>
+      </c>
+      <c r="G10" s="171" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="184" t="n">
+        <v>253.5</v>
+      </c>
+      <c r="I10" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="184" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>490</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>490</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="182" t="n">
+        <v>490</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="182" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="166" t="inlineStr">
+        <is>
+          <t>OUR CHANNEL MIX vs INDUSTRY</t>
+        </is>
+      </c>
+      <c r="B14" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C14" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WeBike web mix [%]</t>
+        </is>
+      </c>
+      <c r="B15" s="179" t="n">
+        <v>0.191</v>
+      </c>
+      <c r="C15" s="170" t="inlineStr">
+        <is>
+          <t>we CUT web staff and spend in Q3</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Industry average web mix [%] (firms with a web centre)</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>0.3492215627413878</v>
+      </c>
+      <c r="C16" s="170" t="inlineStr">
+        <is>
+          <t>MILC 54.4% - LiteCycle 44.2% - BB LLC 37.8% - SpaceBikes 37.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Gap [pct points]</t>
+        </is>
+      </c>
+      <c r="B17" s="10">
+        <f>C16-C15</f>
+        <v/>
+      </c>
+      <c r="C17" s="170" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WeBike web demand [units]</t>
+        </is>
+      </c>
+      <c r="B18" s="167" t="n">
+        <v>120</v>
+      </c>
+      <c r="C18" s="170" t="inlineStr">
+        <is>
+          <t>LOWEST of any firm operating a web centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Industry web demand range</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>138 - 569</t>
+        </is>
+      </c>
+      <c r="C19" s="170" t="inlineStr">
+        <is>
+          <t>Spoke'd Up 138 is the only firm near us</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rank on web demand</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>6 of 7</t>
+        </is>
+      </c>
+      <c r="C20" s="170" t="inlineStr">
+        <is>
+          <t>only Bike Bros is lower, and it has NO web centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="166" t="inlineStr">
+        <is>
+          <t>WHY WEB MATTERS MORE THAN WE THOUGHT</t>
+        </is>
+      </c>
+      <c r="B23" s="166" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C23" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Our demand from New York City (no store)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>38</v>
+      </c>
+      <c r="C24" s="170" t="inlineStr">
+        <is>
+          <t>web only</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Our demand from Bangalore (no store)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="170" t="inlineStr">
+        <is>
+          <t>web only</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Subtotal from cities where we have NO store</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>B24+B25</f>
+        <v/>
+      </c>
+      <c r="C26" s="170" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Total web demand</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>120</v>
+      </c>
+      <c r="C27" s="170" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Share of web demand coming from non-store cities</t>
+        </is>
+      </c>
+      <c r="B28" s="10">
+        <f>B26/B27</f>
+        <v/>
+      </c>
+      <c r="C28" s="170" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Store demand (Amsterdam + Rio)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>507</v>
+      </c>
+      <c r="C29" s="170" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Amsterdam + Rio total demand</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>565</v>
+      </c>
+      <c r="C30" s="170" t="inlineStr">
+        <is>
+          <t>so 58 units of web demand also came from store cities</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>B30-B29</f>
+        <v/>
+      </c>
+      <c r="C31" s="170" t="inlineStr">
+        <is>
+          <t>58 = web demand inside store cities; 58 + 62 = 120 web total</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C32" s="174" t="inlineStr">
+        <is>
+          <t>The web centre is HALF our reach into cities where we have no store. It is the only way to touch New York and Bangalore today, and we shrank it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="166" t="inlineStr">
+        <is>
+          <t>THE WEB REBUILD CASE</t>
+        </is>
+      </c>
+      <c r="B35" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C35" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Current store demand [units]</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>507</v>
+      </c>
+      <c r="C36" s="170" t="inlineStr">
+        <is>
+          <t>hold constant</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Current web demand [units]</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>120</v>
+      </c>
+      <c r="C37" s="170" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Current total</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>B36+B37</f>
+        <v/>
+      </c>
+      <c r="C38" s="170" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>If web mix matched industry average (34.9%)</t>
+        </is>
+      </c>
+      <c r="C39" s="170" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  implied total demand</t>
+        </is>
+      </c>
+      <c r="B40">
+        <f>B36/(1-0.3492)</f>
+        <v/>
+      </c>
+      <c r="C40" s="170" t="inlineStr">
+        <is>
+          <t>store demand becomes 65.1% of total</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  implied web demand</t>
+        </is>
+      </c>
+      <c r="B41">
+        <f>B41-B36</f>
+        <v/>
+      </c>
+      <c r="C41" s="170" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ADDITIONAL demand vs today</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>B42-B37</f>
+        <v/>
+      </c>
+      <c r="C42" s="170" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Contribution per unit (Q3 actual, avg)</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>750</v>
+      </c>
+      <c r="C43" s="170" t="inlineStr">
+        <is>
+          <t>Hike Bike $747 / Swift Bike $756</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Gross margin opportunity</t>
+        </is>
+      </c>
+      <c r="B44">
+        <f>B43*B44</f>
+        <v/>
+      </c>
+      <c r="C44" s="170" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Cost of ~4 additional web staff per quarter</t>
+        </is>
+      </c>
+      <c r="B45" s="159" t="n">
+        <v>24425</v>
+      </c>
+      <c r="C45" s="170" t="inlineStr">
+        <is>
+          <t>$24,425/yr each = ~$6,106/qtr x 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Net quarterly gain</t>
+        </is>
+      </c>
+      <c r="B46">
+        <f>B45-B46</f>
+        <v/>
+      </c>
+      <c r="C46" s="170" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="B47" s="172" t="n"/>
+      <c r="C47" s="170" t="inlineStr">
+        <is>
+          <t>Web headcount is the cheapest demand in the game: no lease, no store setup, and it reaches all four cities. This is a far better first dollar than a third store.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="C48" s="170" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="166" t="inlineStr">
+        <is>
+          <t>STORE PRODUCTIVITY — we under-staff what we own</t>
+        </is>
+      </c>
+      <c r="B50" s="166" t="inlineStr">
+        <is>
+          <t>Demand / store</t>
+        </is>
+      </c>
+      <c r="C50" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>490</v>
+      </c>
+      <c r="C51" s="170" t="inlineStr">
+        <is>
+          <t>ONE store, highest per-store demand in the industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>469</v>
+      </c>
+      <c r="C52" s="170" t="inlineStr">
+        <is>
+          <t>leader</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>404</v>
+      </c>
+      <c r="C53" s="170" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>358</v>
+      </c>
+      <c r="C54" s="170" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>275</v>
+      </c>
+      <c r="C55" s="170" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B56" s="167" t="n">
+        <v>254</v>
+      </c>
+      <c r="C56" s="170" t="inlineStr">
+        <is>
+          <t>LOWEST of the two-store firms</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>364</v>
+      </c>
+      <c r="C57" s="170" t="inlineStr">
+        <is>
+          <t>web-first model; Amsterdam store base</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C58" s="170" t="inlineStr">
+        <is>
+          <t>BB LLC pulls 1.8x our demand from the same number of stores. Depth inside Amsterdam and Rio is unfinished business before we add a third location.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="166" t="inlineStr">
+        <is>
+          <t>CHANNEL MODELS IN THIS INDUSTRY</t>
+        </is>
+      </c>
+      <c r="B61" s="166" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="C61" s="166" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Web-first</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>MILC Bikes - 54.4% web, lowest store demand (364)</t>
+        </is>
+      </c>
+      <c r="C62" s="170" t="inlineStr">
+        <is>
+          <t>12.2% share on 1 store base</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Balanced</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>LiteCycle 44.2% - BB LLC 37.8% - SpaceBikes 37.8%</t>
+        </is>
+      </c>
+      <c r="C63" s="181" t="inlineStr">
+        <is>
+          <t>the three strongest firms sit here</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Store-heavy</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Spoke'd Up 83.8% - WeBike 80.9%</t>
+        </is>
+      </c>
+      <c r="C64" s="170" t="inlineStr">
+        <is>
+          <t>13.0% and 9.6% share</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Store-only</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bike Bros 100% store, no web centre</t>
+        </is>
+      </c>
+      <c r="C65" s="185" t="inlineStr">
+        <is>
+          <t>7.5% share, LAST, falling everywhere</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C66" s="170" t="inlineStr">
+        <is>
+          <t>The top three firms all run 38-44% web. Store-only is last. We are 80.9% store-heavy and drifting toward the Bike Bros failure mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="166" t="inlineStr">
+        <is>
+          <t>Q4 CHANNEL ACTIONS</t>
+        </is>
+      </c>
+      <c r="B69" s="166" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1. Reverse the Q3 web cut</t>
+        </is>
+      </c>
+      <c r="B70" s="174" t="inlineStr">
+        <is>
+          <t>Rehire web sales + support toward 6 people. Cheapest demand available: no lease, no setup, reaches all 4 cities.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2. Restart page upgrades</t>
+        </is>
+      </c>
+      <c r="B71" s="174" t="inlineStr">
+        <is>
+          <t>We stopped this tactic in Q3. Toll-free stayed on. Both were cheap (~$3k and ~$6k/qtr) relative to ~$750 contribution per unit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>3. Deepen Amsterdam + Rio</t>
+        </is>
+      </c>
+      <c r="B72" s="174" t="inlineStr">
+        <is>
+          <t>254 demand/store vs BB LLC's 469. Add store sales staff before adding a third city - same money, faster payback.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>4. Re-evaluate city #3 order</t>
+        </is>
+      </c>
+      <c r="B73" s="174" t="inlineStr">
+        <is>
+          <t>Web already reaches New York (38 units). A store there is still the biggest prize, but web staff + store depth may be the better FIRST dollar this quarter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>5. Never cut channel again</t>
+        </is>
+      </c>
+      <c r="B74" s="174" t="inlineStr">
+        <is>
+          <t>Bike Bros is the control group: 100% store, no web, last place, share falling in all three segments.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Confirm competitor city footprints and correct the Amsterdam read.
The presence report validates every inferred store location and shows MILC runs a
single store. Amsterdam holds all seven rivals, so its low share ceiling reflects
saturation rather than opportunity, and New York carries 579 units per store firm
against Amsterdam's 426. Rio also shows we extract less from a monopoly than
LiteCycle does from the same position.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -38,6 +38,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_City_Demand" sheetId="30" state="visible" r:id="rId30"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_City_Strategy" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Channel" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Presence" sheetId="33" state="visible" r:id="rId33"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -618,7 +619,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="186">
+  <cellXfs count="188">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -883,6 +884,8 @@
     <xf numFmtId="0" fontId="0" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -28597,6 +28600,1066 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" style="146" min="1" max="1"/>
+    <col width="34" customWidth="1" style="146" min="2" max="2"/>
+    <col width="46" customWidth="1" style="146" min="3" max="3"/>
+    <col width="15" customWidth="1" style="146" min="4" max="4"/>
+    <col width="15" customWidth="1" style="146" min="5" max="5"/>
+    <col width="15" customWidth="1" style="146" min="6" max="6"/>
+    <col width="15" customWidth="1" style="146" min="7" max="7"/>
+    <col width="15" customWidth="1" style="146" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Competitors in City — CONFIRMED footprints, Q3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>This report confirms every store location previously INFERRED from demand patterns. One correction: MILC Bikes has only ONE store (Amsterdam), not two.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="I4" s="166" t="inlineStr">
+        <is>
+          <t>Store firms present</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B5" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="C5" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D5" s="173" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E5" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F5" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G5" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H5" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E6" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F6" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G6" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="173" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C8" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Web Sales Centre</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C9" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="D9" s="173" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E9" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F9" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G9" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H9" s="159" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="166" t="inlineStr">
+        <is>
+          <t>CONFIRMED FOOTPRINT</t>
+        </is>
+      </c>
+      <c r="B12" s="166" t="inlineStr">
+        <is>
+          <t>Stores</t>
+        </is>
+      </c>
+      <c r="C12" s="166" t="inlineStr">
+        <is>
+          <t>Cities</t>
+        </is>
+      </c>
+      <c r="D12" s="166" t="inlineStr">
+        <is>
+          <t>Web centre</t>
+        </is>
+      </c>
+      <c r="E12" s="166" t="inlineStr">
+        <is>
+          <t>Total demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Amsterdam, New York City</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Amsterdam, New York City</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Amsterdam, Bangalore</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>984</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Amsterdam, New York City</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="173" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B18" s="173" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="173" t="inlineStr">
+        <is>
+          <t>Amsterdam, Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="D18" s="173" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="E18" s="173" t="n">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D19" s="167" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="166" t="inlineStr">
+        <is>
+          <t>MARKET STRUCTURE — a store never captures the whole city</t>
+        </is>
+      </c>
+      <c r="B22" s="166" t="inlineStr">
+        <is>
+          <t>Store firms</t>
+        </is>
+      </c>
+      <c r="C22" s="166" t="inlineStr">
+        <is>
+          <t>Store-firm demand</t>
+        </is>
+      </c>
+      <c r="D22" s="166" t="inlineStr">
+        <is>
+          <t>Store capture %</t>
+        </is>
+      </c>
+      <c r="E22" s="166" t="inlineStr">
+        <is>
+          <t>Web-only demand</t>
+        </is>
+      </c>
+      <c r="F22" s="166" t="inlineStr">
+        <is>
+          <t>Web-only %</t>
+        </is>
+      </c>
+      <c r="G22" s="166" t="inlineStr">
+        <is>
+          <t>Avg per store firm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>7</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2985</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="186" t="n">
+        <v>426.4285714285714</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1738</v>
+      </c>
+      <c r="D24" s="10" t="n">
+        <v>0.8523786169691026</v>
+      </c>
+      <c r="E24" t="n">
+        <v>301</v>
+      </c>
+      <c r="F24" s="10" t="n">
+        <v>0.1476213830308975</v>
+      </c>
+      <c r="G24" s="187" t="n">
+        <v>579.3333333333334</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>270</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>0.3488372093023256</v>
+      </c>
+      <c r="E25" t="n">
+        <v>504</v>
+      </c>
+      <c r="F25" s="10" t="n">
+        <v>0.6511627906976745</v>
+      </c>
+      <c r="G25" s="182" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>370</v>
+      </c>
+      <c r="D26" s="10" t="n">
+        <v>0.4862023653088042</v>
+      </c>
+      <c r="E26" t="n">
+        <v>391</v>
+      </c>
+      <c r="F26" s="10" t="n">
+        <v>0.5137976346911958</v>
+      </c>
+      <c r="G26" s="182" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="166" t="inlineStr">
+        <is>
+          <t>CORRECTION — Amsterdam is the MOST contested city, not an open one</t>
+        </is>
+      </c>
+      <c r="B29" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Earlier read</t>
+        </is>
+      </c>
+      <c r="B30" s="185" t="inlineStr">
+        <is>
+          <t>'No rival exceeds 16.5%, so Amsterdam is genuinely open.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>What the presence report shows</t>
+        </is>
+      </c>
+      <c r="B31" s="170" t="inlineStr">
+        <is>
+          <t>ALL SEVEN firms hold an Amsterdam store. Nobody exceeds 16.5% precisely BECAUSE all seven are there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Avg demand per store firm - Amsterdam</t>
+        </is>
+      </c>
+      <c r="B32" s="170" t="n">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Avg demand per store firm - New York City</t>
+        </is>
+      </c>
+      <c r="B33" s="170" t="n">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Implication</t>
+        </is>
+      </c>
+      <c r="B34" s="181" t="inlineStr">
+        <is>
+          <t>A store in New York is worth MORE than deeper investment in Amsterdam. Amsterdam is 2,985 units split 7 ways; New York is 2,039 units split 3 ways. Gaining share in Amsterdam means taking it from six store-equipped rivals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="166" t="inlineStr">
+        <is>
+          <t>RIO — we under-exploit our monopoly</t>
+        </is>
+      </c>
+      <c r="B37" s="166" t="inlineStr">
+        <is>
+          <t>WeBike in Rio</t>
+        </is>
+      </c>
+      <c r="C37" s="166" t="inlineStr">
+        <is>
+          <t>LiteCycle in Bangalore</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Only firm with a store in the city</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>City demand</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>774</v>
+      </c>
+      <c r="C39" t="n">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Our / their units</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>270</v>
+      </c>
+      <c r="C40" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Share as sole store holder</t>
+        </is>
+      </c>
+      <c r="B41" s="179" t="n">
+        <v>0.349</v>
+      </c>
+      <c r="C41" s="161" t="n">
+        <v>0.486</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Gap</t>
+        </is>
+      </c>
+      <c r="B42">
+        <f>C41-B41</f>
+        <v/>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>13.7 pts of share we leave on the table</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Web-only rivals take</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>504</v>
+      </c>
+      <c r="C43" t="n">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Web-only rivals' capture %</t>
+        </is>
+      </c>
+      <c r="B44" s="10">
+        <f>B43/B39</f>
+        <v/>
+      </c>
+      <c r="C44" s="10">
+        <f>C43/C39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C45" s="174" t="inlineStr">
+        <is>
+          <t>Same structural position, nearly identical city size - LiteCycle extracts 13.7 more points than we do. Rio opened only in Q3 and we stocked out, so some of this is timing. But 65% of OUR exclusive city still goes to rivals who have no store there at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="166" t="inlineStr">
+        <is>
+          <t>WHY THE WEB CASE IS NOW STRONGER</t>
+        </is>
+      </c>
+      <c r="B48" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="B49" s="170" t="inlineStr">
+        <is>
+          <t>BB LLC pulls 139 units out of Rio with NO store there - 51% of what we get WITH a store. SpaceBikes 120, MILC 107, LiteCycle 106. Web-only rivals took 504 of Rio's 774 units.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Our mirror position</t>
+        </is>
+      </c>
+      <c r="B50" s="170" t="inlineStr">
+        <is>
+          <t>We pull only 38 from New York and 24 from Bangalore by web. Rivals do 3-5x better at the same trick.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Conclusion</t>
+        </is>
+      </c>
+      <c r="B51" s="174" t="inlineStr">
+        <is>
+          <t>Web reach is not a consolation prize for cities we skip - it is how the strong firms raid cities they never entered. Our 19.1% web mix is costing us in all four cities, including the two where we have stores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="166" t="inlineStr">
+        <is>
+          <t>CITY #3 — updated read</t>
+        </is>
+      </c>
+      <c r="B54" s="166" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="C54" s="166" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>City demand</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2039</v>
+      </c>
+      <c r="C55" t="n">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Store firms already present</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Avg demand per store firm today</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>579</v>
+      </c>
+      <c r="C57" t="n">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Weakest incumbent store firm</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Spoke'd Up 412</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Our current web-only demand there</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>38</v>
+      </c>
+      <c r="C59" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Plausible units with a store</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>412 - 574 (match Spoke'd Up or SpaceBikes)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>~250 (split LiteCycle's monopoly)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="B61" s="181" t="inlineStr">
+        <is>
+          <t>STILL THE BEST STORE TARGET. 2.7x the demand, and only 3 rivals hold stores vs Amsterdam's 7. Enter via SPEED (880 units, no dominant firm) - BB LLC holds 82.8% of NYC Mountain.</t>
+        </is>
+      </c>
+      <c r="C61" s="170" t="inlineStr">
+        <is>
+          <t>Smallest prize. LiteCycle's 48.6% monopoly is the industry's most concentrated position.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="166" t="inlineStr">
+        <is>
+          <t>Q4 SEQUENCING — reconciling depth vs breadth</t>
+        </is>
+      </c>
+      <c r="B64" s="166" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1st dollar: web rebuild</t>
+        </is>
+      </c>
+      <c r="B65" s="174" t="inlineStr">
+        <is>
+          <t>Cheapest demand, reaches all 4 cities, pays back in-quarter (~+$89,600). Rivals prove web raids cities you never enter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2nd dollar: Rio depth</t>
+        </is>
+      </c>
+      <c r="B66" s="174" t="inlineStr">
+        <is>
+          <t>We are the ONLY store in Rio and extract just 34.9% vs LiteCycle's 48.6% in the same position. Closing that gap is ~106 units with no new lease.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>3rd dollar: New York store</t>
+        </is>
+      </c>
+      <c r="B67" s="174" t="inlineStr">
+        <is>
+          <t>Biggest single prize (2,039 units, only 3 store rivals). Enter through Speed once Swift Bike is fixed to 77.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>NOT a priority</t>
+        </is>
+      </c>
+      <c r="B68" s="174" t="inlineStr">
+        <is>
+          <t>Deepening Amsterdam against 6 store-equipped rivals; opening Bangalore against LiteCycle's entrenched 48.6%.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Q3 staffing detail and the seven-person city cap.
No firm exceeds seven sales and service people in a city, and Amsterdam already
holds us at that ceiling, so store depth is only available by filling Rio's three
open slots or opening a new city. We also carry two untrained sellers that 800
dollars of training would fix, and our demand per store person is last at 46.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -39,6 +39,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_City_Strategy" sheetId="31" state="visible" r:id="rId31"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Channel" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Presence" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Staffing" sheetId="34" state="visible" r:id="rId34"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -619,7 +620,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="192">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -886,6 +887,10 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="28" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -29660,6 +29665,1611 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J90"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" style="146" min="1" max="1"/>
+    <col width="40" customWidth="1" style="146" min="2" max="2"/>
+    <col width="34" customWidth="1" style="146" min="3" max="3"/>
+    <col width="30" customWidth="1" style="146" min="4" max="4"/>
+    <col width="13" customWidth="1" style="146" min="5" max="5"/>
+    <col width="13" customWidth="1" style="146" min="6" max="6"/>
+    <col width="13" customWidth="1" style="146" min="7" max="7"/>
+    <col width="13" customWidth="1" style="146" min="8" max="8"/>
+    <col width="13" customWidth="1" style="146" min="9" max="9"/>
+    <col width="13" customWidth="1" style="146" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Sales and Service People — World Market, Q3 actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Two hard findings: 7 people per city is the cap (nobody exceeds it, and Amsterdam has us AT it), and we are the only firm besides Bike Bros carrying UNTRAINED staff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>Assigned</t>
+        </is>
+      </c>
+      <c r="I4" s="166" t="inlineStr">
+        <is>
+          <t>UNTRAINED</t>
+        </is>
+      </c>
+      <c r="J4" s="166" t="inlineStr">
+        <is>
+          <t>At 7-cap?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>7</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>New York City</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" t="n">
+        <v>7</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="171" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="B8" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C8" s="171" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="171" t="n">
+        <v>3</v>
+      </c>
+      <c r="I8" s="188" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="171" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I9" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="171" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B11" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C11" s="171" t="n">
+        <v>7</v>
+      </c>
+      <c r="D11" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="171" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="171" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="171" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="188" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="171" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>7</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>7</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" t="n">
+        <v>7</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Bangalore</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>5</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="166" t="inlineStr">
+        <is>
+          <t>FIRM ROLLUP</t>
+        </is>
+      </c>
+      <c r="B19" s="166" t="inlineStr">
+        <is>
+          <t>Store people</t>
+        </is>
+      </c>
+      <c r="C19" s="166" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D19" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="E19" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="F19" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G19" s="166" t="inlineStr">
+        <is>
+          <t>Untrained</t>
+        </is>
+      </c>
+      <c r="H19" s="166" t="inlineStr">
+        <is>
+          <t>Store demand</t>
+        </is>
+      </c>
+      <c r="I19" s="166" t="inlineStr">
+        <is>
+          <t>Demand / store person</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>7</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>490</v>
+      </c>
+      <c r="I20" s="189" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>14</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" t="n">
+        <v>6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>938</v>
+      </c>
+      <c r="I21" s="189" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>11</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>5</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>716</v>
+      </c>
+      <c r="I22" s="189" t="n">
+        <v>65.09090909090909</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>14</v>
+      </c>
+      <c r="C23" t="n">
+        <v>4</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>807</v>
+      </c>
+      <c r="I23" s="189" t="n">
+        <v>57.64285714285715</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" t="n">
+        <v>6</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>549</v>
+      </c>
+      <c r="I24" s="189" t="n">
+        <v>54.9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>3</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>364</v>
+      </c>
+      <c r="I25" s="189" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B26" s="171" t="n">
+        <v>11</v>
+      </c>
+      <c r="C26" s="171" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="171" t="n">
+        <v>4</v>
+      </c>
+      <c r="F26" s="171" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="171" t="n">
+        <v>507</v>
+      </c>
+      <c r="I26" s="190" t="n">
+        <v>46.09090909090909</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="166" t="inlineStr">
+        <is>
+          <t>PRODUCTIVITY GAP</t>
+        </is>
+      </c>
+      <c r="B29" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C29" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>WeBike demand per store person</t>
+        </is>
+      </c>
+      <c r="B30" s="191" t="n">
+        <v>46.09090909090909</v>
+      </c>
+      <c r="C30" s="170" t="inlineStr">
+        <is>
+          <t>LOWEST in the industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Industry average (excl. us)</t>
+        </is>
+      </c>
+      <c r="B31" s="160" t="n">
+        <v>61.1056277056277</v>
+      </c>
+      <c r="C31" s="170" t="inlineStr">
+        <is>
+          <t>Bike Bros 70.0 is best; BB LLC 67.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Shortfall per person</t>
+        </is>
+      </c>
+      <c r="B32" s="189">
+        <f>C31-C30</f>
+        <v/>
+      </c>
+      <c r="C32" s="170" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Our store people</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>11</v>
+      </c>
+      <c r="C33" s="170" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Store demand if we matched the average</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>C31*C33</f>
+        <v/>
+      </c>
+      <c r="C34" s="170" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Additional units available at current headcount</t>
+        </is>
+      </c>
+      <c r="B35" s="159">
+        <f>C34-507</f>
+        <v/>
+      </c>
+      <c r="C35" s="170" t="inlineStr">
+        <is>
+          <t>no new hires needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="166" t="inlineStr">
+        <is>
+          <t>THE 7-PERSON CITY CAP — this settles depth vs breadth</t>
+        </is>
+      </c>
+      <c r="B38" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C38" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Maximum staff observed in any city (all 12 rows)</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>7</v>
+      </c>
+      <c r="C39" s="170" t="inlineStr">
+        <is>
+          <t>BB LLC, SpaceBikes, Bike Bros, MILC and our own Amsterdam all sit at 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>WeBike Amsterdam headcount</t>
+        </is>
+      </c>
+      <c r="B40" s="167" t="n">
+        <v>7</v>
+      </c>
+      <c r="C40" s="170" t="inlineStr">
+        <is>
+          <t>AT THE CAP - we cannot add a single person there</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>WeBike Rio headcount</t>
+        </is>
+      </c>
+      <c r="B41" s="159" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" s="170" t="inlineStr">
+        <is>
+          <t>3 SLOTS OPEN - the only store depth available to us</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C42" s="174" t="inlineStr">
+        <is>
+          <t>'Deepen Amsterdam' is not a legal move. Amsterdam is maxed at 7. The only ways to add store selling capacity are (a) fill Rio's 3 open slots, or (b) open a new city, which unlocks 7 more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="166" t="inlineStr">
+        <is>
+          <t>RIO vs AMSTERDAM — where a body is worth more</t>
+        </is>
+      </c>
+      <c r="B45" s="166" t="inlineStr">
+        <is>
+          <t>Rio</t>
+        </is>
+      </c>
+      <c r="C45" s="166" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Store people</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>4</v>
+      </c>
+      <c r="C46" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>City demand (all channels)</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>270</v>
+      </c>
+      <c r="C47" t="n">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Demand per person</t>
+        </is>
+      </c>
+      <c r="B48" s="160">
+        <f>C47/C46</f>
+        <v/>
+      </c>
+      <c r="C48" s="191">
+        <f>D47/D46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Rival stores in city</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Open slots to the 7-cap</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>3</v>
+      </c>
+      <c r="C50" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="B51" s="174" t="inlineStr">
+        <is>
+          <t>A Rio head is worth ~60% more than an Amsterdam head because Rio has no rival store. Filling the 3 open Rio slots is the highest-return staffing move on the board.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>CAVEAT</t>
+        </is>
+      </c>
+      <c r="B52" s="170" t="inlineStr">
+        <is>
+          <t>City demand includes web orders, so per-person figures are directional rather than pure store productivity. The ranking is robust; the exact multiple is not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="166" t="inlineStr">
+        <is>
+          <t>UNTRAINED STAFF — a free win we skipped</t>
+        </is>
+      </c>
+      <c r="B55" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C55" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>WeBike untrained people</t>
+        </is>
+      </c>
+      <c r="B56" s="167" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" s="170" t="inlineStr">
+        <is>
+          <t>1 in Rio, 1 in Amsterdam</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Firms with any untrained staff</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>WeBike (2), Bike Bros (1)</t>
+        </is>
+      </c>
+      <c r="C57" s="170" t="inlineStr">
+        <is>
+          <t>the other five are 100% trained</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Mountain training cost</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>400</v>
+      </c>
+      <c r="C58" s="170" t="inlineStr">
+        <is>
+          <t>per quarter</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Speed training cost</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>400</v>
+      </c>
+      <c r="C59" s="170" t="inlineStr">
+        <is>
+          <t>per quarter</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Cost to train both</t>
+        </is>
+      </c>
+      <c r="B60" s="159" t="n">
+        <v>800</v>
+      </c>
+      <c r="C60" s="170" t="inlineStr">
+        <is>
+          <t>trivial against ~$750 contribution PER UNIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C61" s="174" t="inlineStr">
+        <is>
+          <t>We are paying two full salaries ($24,425/yr each) for untrained sellers while every serious competitor trains everyone. Fix this first - it costs $800.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="166" t="inlineStr">
+        <is>
+          <t>SPECIALISATION vs SEGMENT RESULT</t>
+        </is>
+      </c>
+      <c r="B64" s="166" t="inlineStr">
+        <is>
+          <t>Specialists</t>
+        </is>
+      </c>
+      <c r="C64" s="166" t="inlineStr">
+        <is>
+          <t>Segment demand</t>
+        </is>
+      </c>
+      <c r="D64" s="166" t="inlineStr">
+        <is>
+          <t>Demand per specialist</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="166" t="inlineStr">
+        <is>
+          <t>MOUNTAIN</t>
+        </is>
+      </c>
+      <c r="D65" s="189" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="n">
+        <v>340</v>
+      </c>
+      <c r="D66" s="189">
+        <f>C66/B66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>6</v>
+      </c>
+      <c r="C67" t="n">
+        <v>751</v>
+      </c>
+      <c r="D67" s="189">
+        <f>C67/B67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="173" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="n">
+        <v>358</v>
+      </c>
+      <c r="D68" s="189">
+        <f>C68/B68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="n">
+        <v>172</v>
+      </c>
+      <c r="D69" s="189">
+        <f>C69/B69</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="166" t="inlineStr">
+        <is>
+          <t>SPEED</t>
+        </is>
+      </c>
+      <c r="D70" s="189" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>6</v>
+      </c>
+      <c r="C71" t="n">
+        <v>657</v>
+      </c>
+      <c r="D71" s="189">
+        <f>C71/B71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n">
+        <v>328</v>
+      </c>
+      <c r="D72" s="189">
+        <f>C72/B72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>6</v>
+      </c>
+      <c r="C73" t="n">
+        <v>588</v>
+      </c>
+      <c r="D73" s="189">
+        <f>C73/B73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>6</v>
+      </c>
+      <c r="C74" t="n">
+        <v>548</v>
+      </c>
+      <c r="D74" s="189">
+        <f>C74/B74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" t="n">
+        <v>362</v>
+      </c>
+      <c r="D75" s="189">
+        <f>C75/B75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="173" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B76" s="167" t="n">
+        <v>3</v>
+      </c>
+      <c r="C76" t="n">
+        <v>215</v>
+      </c>
+      <c r="D76" s="189">
+        <f>C76/B76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="166" t="inlineStr">
+        <is>
+          <t>RECREATION</t>
+        </is>
+      </c>
+      <c r="D77" s="189" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>4</v>
+      </c>
+      <c r="C78" t="n">
+        <v>710</v>
+      </c>
+      <c r="D78" s="189">
+        <f>C78/B78</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>3</v>
+      </c>
+      <c r="C79" t="n">
+        <v>471</v>
+      </c>
+      <c r="D79" s="189">
+        <f>C79/B79</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>4</v>
+      </c>
+      <c r="C80" t="n">
+        <v>492</v>
+      </c>
+      <c r="D80" s="189">
+        <f>C80/B80</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="173" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>0</v>
+      </c>
+      <c r="C81" t="n">
+        <v>54</v>
+      </c>
+      <c r="D81" s="189" t="inlineStr">
+        <is>
+          <t>spillover only - no Rec specialists</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="166" t="inlineStr">
+        <is>
+          <t>Q4 STAFFING PLAN</t>
+        </is>
+      </c>
+      <c r="B84" s="166" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C84" s="166" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="D84" s="166" t="inlineStr">
+        <is>
+          <t>Expected units</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1. Train the 2 untrained</t>
+        </is>
+      </c>
+      <c r="B85" s="174" t="inlineStr">
+        <is>
+          <t>1 Mountain (Rio) + 1 Speed (Amsterdam)</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>800</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>free productivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2. Fill Rio to the 7-cap</t>
+        </is>
+      </c>
+      <c r="B86" s="174" t="inlineStr">
+        <is>
+          <t>+3 people: 1 Mountain, 1 Speed, 1 Service</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>~$18,300/qtr salary + hire + train</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>~+200 at Rio's ~67/head</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>3. Rebuild web staff</t>
+        </is>
+      </c>
+      <c r="B87" s="174" t="inlineStr">
+        <is>
+          <t>3 -&gt; 6 web sales/support</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>~$18,300/qtr</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>~+152 (see Q3_Channel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>4. Add Speed specialists</t>
+        </is>
+      </c>
+      <c r="B88" s="174" t="inlineStr">
+        <is>
+          <t>we have 3 vs BB LLC/LiteCycle/SpaceBikes 6</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>included above</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Speed is our weakest segment AND the largest</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>5. New York store (if funded)</t>
+        </is>
+      </c>
+      <c r="B89" s="174" t="inlineStr">
+        <is>
+          <t>unlocks 7 fresh slots; staff Speed-heavy</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>setup + lease + salaries</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>~400-570 at incumbent rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>NOT possible</t>
+        </is>
+      </c>
+      <c r="B90" s="185" t="inlineStr">
+        <is>
+          <t>Adding anyone in Amsterdam - we are at the 7-person cap</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Q3 web operations and correct the capacity formula.
Web staff shares the seven-person cap and we run three, while only one of four web
productivity tactics is funded; every firm funding all four reaches 435 to 569 web
units against our 120. Also fix the planner's operating-capacity formula to divide
by productivity, which shows Rio plus the web rebuild now exceeds our 24 per day.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -40,6 +40,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Channel" sheetId="32" state="visible" r:id="rId32"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Presence" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Staffing" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Web_Ops" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -52,7 +53,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -242,6 +243,10 @@
     <font>
       <b val="1"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="34">
@@ -620,7 +625,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="192">
+  <cellXfs count="193">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -891,6 +896,7 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="28" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18169,7 +18175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="146" min="1" max="1"/>
@@ -18188,7 +18194,7 @@
     <row r="2">
       <c r="A2" s="170" t="inlineStr">
         <is>
-          <t>Rule: OC/day = forecast demand / 65 * (1 + (1 - productivity)). Never schedule below forecast again. Q3 proof: OC 8/day vs 24 owned -&gt; 204 stock-outs AND labor cost/unit up $130-&gt;$205.</t>
+          <t>Rule: required OC/day = forecast units / (productivity x 65 days). Never schedule below the forecast again. Q3 proof: OC 8/day vs 24 owned -&gt; 204 stock-outs AND labour cost/unit up $130 -&gt; $205.</t>
         </is>
       </c>
     </row>
@@ -18288,12 +18294,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Productivity pad</t>
-        </is>
-      </c>
-      <c r="B9">
-        <f>1+(1-B8)</f>
-        <v/>
+          <t>Capacity factor (1 / productivity)</t>
+        </is>
+      </c>
+      <c r="B9" s="159">
+        <f>1/B8</f>
+        <v/>
+      </c>
+      <c r="C9" s="170" t="inlineStr">
+        <is>
+          <t>CORRECTED: was 1+(1-p)=1.26, which understated the requirement. 1/0.74 = 1.35.</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -18303,12 +18314,12 @@
         </is>
       </c>
       <c r="B10">
-        <f>B7/65*B9</f>
+        <f>B7/(B8*65)</f>
         <v/>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>schedule AT LEAST this</t>
+          <t>units / (productivity x days) - schedule AT LEAST this</t>
         </is>
       </c>
     </row>
@@ -18795,46 +18806,431 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Q4 forecast units</t>
-        </is>
-      </c>
-      <c r="B46">
-        <f>B7</f>
-        <v/>
+      <c r="A46" s="166" t="inlineStr">
+        <is>
+          <t>DEMAND SCENARIOS -&gt; REQUIRED OPERATING CAPACITY</t>
+        </is>
+      </c>
+      <c r="B46" s="166" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="C46" s="166" t="inlineStr">
+        <is>
+          <t>Required OC/day</t>
+        </is>
+      </c>
+      <c r="D46" s="166" t="inlineStr">
+        <is>
+          <t>Fits in 24/day?</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>COGS saving on forecast volume</t>
-        </is>
-      </c>
-      <c r="B47">
-        <f>B45*B46</f>
+          <t>A. Do nothing (Q3 demand less 16.3% ill will)</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>525</v>
+      </c>
+      <c r="C47" s="189">
+        <f>B48/(0.74*65)</f>
+        <v/>
+      </c>
+      <c r="D47">
+        <f>IF(C48&lt;=24,"yes","NO")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>+ Gross margin recovered from ending stock-outs</t>
+          <t>B. Base forecast (planner B7)</t>
         </is>
       </c>
       <c r="B48">
-        <f>Q3_Unit_Economics!I6</f>
+        <f>B7</f>
+        <v/>
+      </c>
+      <c r="C48" s="189">
+        <f>B49/(0.74*65)</f>
+        <v/>
+      </c>
+      <c r="D48">
+        <f>IF(C49&lt;=24,"yes","NO")</f>
         <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49">
-        <f> Combined Q4 swing vs Q3 behaviour</f>
-        <v/>
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>C. + fill Rio to the 7-person cap</t>
+        </is>
       </c>
       <c r="B49" s="159">
-        <f>B47+B48</f>
-        <v/>
+        <f>B49+200</f>
+        <v/>
+      </c>
+      <c r="C49" s="189">
+        <f>B50/(0.74*65)</f>
+        <v/>
+      </c>
+      <c r="D49">
+        <f>IF(C50&lt;=24,"yes","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>D. + full web rebuild (7 staff, 4 tactics)</t>
+        </is>
+      </c>
+      <c r="B50">
+        <f>B50+315</f>
+        <v/>
+      </c>
+      <c r="C50" s="189">
+        <f>B51/(0.74*65)</f>
+        <v/>
+      </c>
+      <c r="D50">
+        <f>IF(C51&lt;=24,"yes","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>E. + New York store</t>
+        </is>
+      </c>
+      <c r="B51">
+        <f>B51+400</f>
+        <v/>
+      </c>
+      <c r="C51" s="189">
+        <f>B52/(0.74*65)</f>
+        <v/>
+      </c>
+      <c r="D51" s="167">
+        <f>IF(C52&lt;=24,"yes","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Max units at 24/day and 74% productivity</t>
+        </is>
+      </c>
+      <c r="B52" s="159">
+        <f>24*0.74*65</f>
+        <v/>
+      </c>
+      <c r="D52" s="167" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D53" s="185" t="inlineStr">
+        <is>
+          <t>Scenario C (Rio fill) fits comfortably at 17.8/day. Scenario D (Rio + full web rebuild) needs 24.3/day and EXCEEDS our 24/day fixed capacity by a hair. Scenario E (plus New York) needs 32.7/day. Capacity - not demand, not product - is now the binding constraint on growth.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="166" t="inlineStr">
+        <is>
+          <t>WEB &amp; STAFFING TARGETS (from Q3_Web_Ops / Q3_Staffing)</t>
+        </is>
+      </c>
+      <c r="B56" s="166" t="inlineStr">
+        <is>
+          <t>WeBike Q3</t>
+        </is>
+      </c>
+      <c r="C56" s="166" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="D56" s="166" t="inlineStr">
+        <is>
+          <t>Q4 target</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Web staff (cap is 7)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>3</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>7 (four firms)</t>
+        </is>
+      </c>
+      <c r="D57" s="168" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Web productivity tactics funded (of 4)</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+      <c r="C58" t="n">
+        <v>4</v>
+      </c>
+      <c r="D58" s="168" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Web productivity budget</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>24,000 - 33,000</t>
+        </is>
+      </c>
+      <c r="D59" s="168" t="n">
+        <v>28000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Web demand</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>120</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>435 - 569</t>
+        </is>
+      </c>
+      <c r="D60" s="168" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Rio store staff (cap is 7)</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="168" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Amsterdam store staff (cap is 7)</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>7</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D62" s="168" t="inlineStr">
+        <is>
+          <t>7 (AT CAP - no room)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Untrained staff</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2</v>
+      </c>
+      <c r="C63" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="167" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="166" t="inlineStr">
+        <is>
+          <t>CAPACITY IS NOW THE BINDING CONSTRAINT — and idle cash is the cure</t>
+        </is>
+      </c>
+      <c r="B66" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C66" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Cash sitting idle</t>
+        </is>
+      </c>
+      <c r="B67" s="167" t="n">
+        <v>1010838</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>the direct cause of Asset Management 0.353 (LAST place)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Fixed capacity today</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>24</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>3 printers, $720,000 original cost -&gt; ~$240,000 each</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Max units at 24/day and 74% productivity</t>
+        </is>
+      </c>
+      <c r="B69">
+        <f>24*0.74*65</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Demand if we fill Rio AND rebuild web</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1171</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>exceeds the ceiling by ~17 units</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>A 4th printer would give</t>
+        </is>
+      </c>
+      <c r="B71" s="159" t="n">
+        <v>32</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>units/day -&gt; max ~1,539 units</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Approx capital cost</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>240000</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>24% of idle cash</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Approx added depreciation</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>per quarter</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C74" s="174" t="inlineStr">
+        <is>
+          <t>Buying capacity solves TWO problems at once: it lifts the growth ceiling AND converts idle cash into revenue-producing assets, which is exactly what Asset Management 0.353 is punishing. Note that owning capacity is NOT what caused Q2's $148,652 excess-capacity charge - that came from SCHEDULING operating capacity we did not use. Depreciation is the only carrying cost of ownership.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Decision framing</t>
+        </is>
+      </c>
+      <c r="C75" s="174" t="inlineStr">
+        <is>
+          <t>If we want Rio + web + New York we need roughly 33/day, i.e. 2 more printers. If we want Rio + web only, 1 more printer gives comfortable slack. Doing nothing caps us at ~1,154 units.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -29822,7 +30218,6 @@
       <c r="I6" t="n">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -29966,7 +30361,6 @@
       <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="171" t="inlineStr">
@@ -30076,7 +30470,6 @@
       <c r="I13" t="n">
         <v>0</v>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -30186,7 +30579,6 @@
       <c r="I16" t="n">
         <v>0</v>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="166" t="inlineStr">
@@ -31262,6 +31654,1134 @@
       <c r="B90" s="185" t="inlineStr">
         <is>
           <t>Adding anyone in Amsterdam - we are at the 7-person cap</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="50" customWidth="1" style="146" min="1" max="1"/>
+    <col width="16" customWidth="1" style="146" min="2" max="2"/>
+    <col width="20" customWidth="1" style="146" min="3" max="3"/>
+    <col width="58" customWidth="1" style="146" min="4" max="4"/>
+    <col width="14" customWidth="1" style="146" min="5" max="5"/>
+    <col width="14" customWidth="1" style="146" min="6" max="6"/>
+    <col width="14" customWidth="1" style="146" min="7" max="7"/>
+    <col width="14" customWidth="1" style="146" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Web Sales &amp; Service + Web Productivity Budgets — Q3 actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Two findings: web staff is ALSO capped at 7 and we sit at 3, and there are FOUR web productivity tactics of which we fund ONE. Every firm running all four gets 435-569 web units; the two running fewer get 120-138.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>WEB STAFF</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Web demand</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Demand / web head</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Slots open to 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" t="n">
+        <v>569</v>
+      </c>
+      <c r="F5" s="189" t="n">
+        <v>81.28571428571429</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>491</v>
+      </c>
+      <c r="F6" s="189" t="n">
+        <v>70.14285714285714</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" t="n">
+        <v>435</v>
+      </c>
+      <c r="F7" s="189" t="n">
+        <v>62.14285714285715</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>435</v>
+      </c>
+      <c r="F8" s="189" t="n">
+        <v>62.14285714285715</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>138</v>
+      </c>
+      <c r="F9" s="189" t="n">
+        <v>46</v>
+      </c>
+      <c r="G9" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B10" s="171" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="171" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="171" t="n">
+        <v>120</v>
+      </c>
+      <c r="F10" s="190" t="n">
+        <v>40</v>
+      </c>
+      <c r="G10" s="188" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="189" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>no web centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="166" t="inlineStr">
+        <is>
+          <t>THE WEB STAFF CAP</t>
+        </is>
+      </c>
+      <c r="B14" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C14" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Max web staff observed</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="170" t="inlineStr">
+        <is>
+          <t>LiteCycle, BB LLC, SpaceBikes and MILC all sit exactly at 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WeBike web staff</t>
+        </is>
+      </c>
+      <c r="B16" s="167" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="170" t="inlineStr">
+        <is>
+          <t>2 sales + 1 service - we CUT to this in Q3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Slots open</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" s="170" t="inlineStr">
+        <is>
+          <t>same 7-person ceiling as the city stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Our demand per web head</t>
+        </is>
+      </c>
+      <c r="B18" s="167" t="n">
+        <v>40</v>
+      </c>
+      <c r="C18" s="170" t="inlineStr">
+        <is>
+          <t>LOWEST of all six firms with a web centre</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Leader demand per web head</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>81.3</v>
+      </c>
+      <c r="C19" s="170" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C20" s="174" t="inlineStr">
+        <is>
+          <t>The web centre has the same 7-person ceiling as a store, but unlike Amsterdam we are nowhere near it. Four open slots and the worst output per head is the largest single pool of unclaimed demand we have found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="166" t="inlineStr">
+        <is>
+          <t>WEB PRODUCTIVITY BUDGETS</t>
+        </is>
+      </c>
+      <c r="B23" s="166" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C23" s="166" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="D23" s="166" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="E23" s="166" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="F23" s="166" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="G23" s="166" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="H23" s="166" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Toll-free phone advising / service calls</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C24" s="171" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D24" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E24" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F24" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G24" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H24" t="n">
+        <v>5667</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Advanced shopping cart &amp; checkout</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C25" s="188" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>7000</v>
+      </c>
+      <c r="G25" t="n">
+        <v>7000</v>
+      </c>
+      <c r="H25" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Continuous page upgrades (content, appeal, navigation)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C26" s="188" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F26" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="H26" t="n">
+        <v>6667</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Order tracking software</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C27" s="188" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>8000</v>
+      </c>
+      <c r="G27" t="n">
+        <v>8000</v>
+      </c>
+      <c r="H27" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>29000</v>
+      </c>
+      <c r="C28" s="171" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D28" t="n">
+        <v>33000</v>
+      </c>
+      <c r="E28" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F28" t="n">
+        <v>33000</v>
+      </c>
+      <c r="G28" t="n">
+        <v>24000</v>
+      </c>
+      <c r="H28" t="n">
+        <v>27334</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Tactics funded (of 4)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" t="n">
+        <v>4</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Web demand</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>435</v>
+      </c>
+      <c r="C30" s="171" t="n">
+        <v>120</v>
+      </c>
+      <c r="D30" t="n">
+        <v>569</v>
+      </c>
+      <c r="E30" t="n">
+        <v>138</v>
+      </c>
+      <c r="F30" t="n">
+        <v>491</v>
+      </c>
+      <c r="G30" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="166" t="inlineStr">
+        <is>
+          <t>THE PATTERN IS ALMOST PERFECT</t>
+        </is>
+      </c>
+      <c r="B33" s="166" t="inlineStr">
+        <is>
+          <t>Tactics funded</t>
+        </is>
+      </c>
+      <c r="C33" s="166" t="inlineStr">
+        <is>
+          <t>Total budget</t>
+        </is>
+      </c>
+      <c r="D33" s="166" t="inlineStr">
+        <is>
+          <t>Web demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>4</v>
+      </c>
+      <c r="C34" t="n">
+        <v>33000</v>
+      </c>
+      <c r="D34" s="159" t="n">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n">
+        <v>33000</v>
+      </c>
+      <c r="D35" s="159" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n">
+        <v>29000</v>
+      </c>
+      <c r="D36" s="159" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n">
+        <v>24000</v>
+      </c>
+      <c r="D37" s="159" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D38" s="167" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D39" s="167" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D40" s="174" t="inlineStr">
+        <is>
+          <t>Every firm funding all four tactics ($24k-33k) lands at 435-569 web units. Both firms funding fewer land at 120-138. Headcount moves with budget (7 vs 3) so the two effects cannot be fully separated - but we are at the bottom of BOTH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="166" t="inlineStr">
+        <is>
+          <t>WHAT WE NEVER STARTED</t>
+        </is>
+      </c>
+      <c r="B43" s="166" t="inlineStr">
+        <is>
+          <t>Our budget</t>
+        </is>
+      </c>
+      <c r="C43" s="166" t="inlineStr">
+        <is>
+          <t>Industry average</t>
+        </is>
+      </c>
+      <c r="D43" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Toll-free phone</t>
+        </is>
+      </c>
+      <c r="B44" s="159" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C44" t="n">
+        <v>5667</v>
+      </c>
+      <c r="D44" s="170" t="inlineStr">
+        <is>
+          <t>ABOVE average - our one good web decision (raised from $3k)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Advanced shopping cart &amp; checkout</t>
+        </is>
+      </c>
+      <c r="B45" s="167" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" t="n">
+        <v>7000</v>
+      </c>
+      <c r="D45" s="170" t="inlineStr">
+        <is>
+          <t>NEVER STARTED - 4 of 6 firms fund it at $7,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Continuous page upgrades</t>
+        </is>
+      </c>
+      <c r="B46" s="167" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" t="n">
+        <v>6667</v>
+      </c>
+      <c r="D46" s="170" t="inlineStr">
+        <is>
+          <t>WE STOPPED THIS IN Q3 - SpaceBikes funds it at $12,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Order tracking software</t>
+        </is>
+      </c>
+      <c r="B47" s="167" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D47" s="170" t="inlineStr">
+        <is>
+          <t>NEVER STARTED - 4 of 6 firms fund it at $8,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Our total</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C48" t="n">
+        <v>27500</v>
+      </c>
+      <c r="D48" s="170" t="inlineStr">
+        <is>
+          <t>average of the four full-tactic firms</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="166" t="inlineStr">
+        <is>
+          <t>THE FULL WEB REBUILD CASE</t>
+        </is>
+      </c>
+      <c r="B51" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C51" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Current web demand</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>120</v>
+      </c>
+      <c r="C52" s="170" t="inlineStr">
+        <is>
+          <t>3 staff, 1 tactic, $6,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Full-tactic cohort web demand range</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>435 - 569</t>
+        </is>
+      </c>
+      <c r="C53" s="170" t="inlineStr">
+        <is>
+          <t>7 staff, 4 tactics, $24k-33k</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Conservative target (cohort floor)</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>435</v>
+      </c>
+      <c r="C54" s="170" t="inlineStr">
+        <is>
+          <t>LiteCycle / MILC level</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Additional demand</t>
+        </is>
+      </c>
+      <c r="B55">
+        <f>C54-C52</f>
+        <v/>
+      </c>
+      <c r="C55" s="170" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Contribution per unit</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>750</v>
+      </c>
+      <c r="C56" s="170" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Gross margin opportunity</t>
+        </is>
+      </c>
+      <c r="B57" s="159">
+        <f>C55*C56</f>
+        <v/>
+      </c>
+      <c r="C57" s="170" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Cost: +4 web staff per quarter</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>24425</v>
+      </c>
+      <c r="C58" s="170" t="inlineStr">
+        <is>
+          <t>4 x $24,425/yr = ~$6,106/qtr each</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Cost: raise web budget $6,000 -&gt; $28,000</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>22000</v>
+      </c>
+      <c r="C59" s="170" t="inlineStr">
+        <is>
+          <t>add 3 tactics, top up toll-free</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Total incremental cost</t>
+        </is>
+      </c>
+      <c r="B60">
+        <f>C58+C59</f>
+        <v/>
+      </c>
+      <c r="C60" s="170" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>NET QUARTERLY GAIN</t>
+        </is>
+      </c>
+      <c r="B61" s="192">
+        <f>C57-C60</f>
+        <v/>
+      </c>
+      <c r="C61" s="170" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="C62" s="170" t="inlineStr">
+        <is>
+          <t>This supersedes the earlier +$89,600 estimate, which only modelled matching the average web MIX. Matching the leaders' web OPERATION is worth far more.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="166" t="inlineStr">
+        <is>
+          <t>CAPACITY WARNING</t>
+        </is>
+      </c>
+      <c r="B65" s="166" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="C65" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Store demand today</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>507</v>
+      </c>
+      <c r="C66" s="170" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Rio +3 staff at ~67/head</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>200</v>
+      </c>
+      <c r="C67" s="170" t="inlineStr">
+        <is>
+          <t>see Q3_Staffing</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Web at cohort floor</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>435</v>
+      </c>
+      <c r="C68" s="170" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Indicative total demand</t>
+        </is>
+      </c>
+      <c r="B69">
+        <f>C66+C67+C68</f>
+        <v/>
+      </c>
+      <c r="C69" s="170" t="inlineStr">
+        <is>
+          <t>before ill will</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Max units at 24/day, 65 days, 74% productivity</t>
+        </is>
+      </c>
+      <c r="B70">
+        <f>24*65*0.74</f>
+        <v/>
+      </c>
+      <c r="C70" s="170" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Required scheduled OC per day</t>
+        </is>
+      </c>
+      <c r="B71" s="168">
+        <f>C69/(0.74*65)</f>
+        <v/>
+      </c>
+      <c r="C71" s="170" t="inlineStr">
+        <is>
+          <t>units / (productivity x days)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Fixed capacity per day</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>24</v>
+      </c>
+      <c r="C72" s="170" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Headroom</t>
+        </is>
+      </c>
+      <c r="B73">
+        <f>C72-C71</f>
+        <v/>
+      </c>
+      <c r="C73" s="170" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C74" s="174" t="inlineStr">
+        <is>
+          <t>Doing all of this at once pushes demand toward ~1,140 and required OC to roughly 21/day - inside our 24/day fixed capacity, but with little slack. Schedule OC to the FORECAST and re-run the production simulation before committing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Q3 price judgment and derive rival price tiers.
Identical judgment triplets imply identical prices, which ranks every competitor's
price without the price list. Hike Bike already sits at the highest tier that draws
no Mountain resistance, while Speed tolerates prices one to two tiers above Swift
Bike, and BB LLC's Mountain brand matches ours on product and price alike.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -41,6 +41,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Presence" sheetId="33" state="visible" r:id="rId33"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Staffing" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Web_Ops" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Price_Judgment" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -625,7 +626,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="193">
+  <cellXfs count="194">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -897,6 +898,9 @@
     <xf numFmtId="165" fontId="28" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32790,6 +32794,1691 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H96"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" style="146" min="1" max="1"/>
+    <col width="22" customWidth="1" style="146" min="2" max="2"/>
+    <col width="30" customWidth="1" style="146" min="3" max="3"/>
+    <col width="60" customWidth="1" style="146" min="4" max="4"/>
+    <col width="56" customWidth="1" style="146" min="5" max="5"/>
+    <col width="16" customWidth="1" style="146" min="6" max="6"/>
+    <col width="16" customWidth="1" style="146" min="7" max="7"/>
+    <col width="16" customWidth="1" style="146" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Price Judgment — World Market, Q3 actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>100 = no price resistance. Lower = buyers find the price high. Because the score depends only on price vs segment willingness-to-pay, identical triplets imply identical prices - which lets us rank every rival's price without seeing the price list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Price judgment in target</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>Resistance?</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>63</v>
+      </c>
+      <c r="D5" t="n">
+        <v>78</v>
+      </c>
+      <c r="E5" t="n">
+        <v>90</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G5" s="167" t="n">
+        <v>90</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>73</v>
+      </c>
+      <c r="D6" t="n">
+        <v>91</v>
+      </c>
+      <c r="E6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G6" s="167" t="n">
+        <v>91</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-9</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mach 0.6</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D7" t="n">
+        <v>86</v>
+      </c>
+      <c r="E7" t="n">
+        <v>100</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G7" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>TERRAMean</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>82</v>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G8" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MountainCruise1</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>92</v>
+      </c>
+      <c r="D9" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" t="n">
+        <v>100</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G9" s="167" t="n">
+        <v>92</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>73</v>
+      </c>
+      <c r="D10" t="n">
+        <v>90</v>
+      </c>
+      <c r="E10" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G10" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>83</v>
+      </c>
+      <c r="D11" t="n">
+        <v>100</v>
+      </c>
+      <c r="E11" t="n">
+        <v>100</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G11" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>85</v>
+      </c>
+      <c r="D12" t="n">
+        <v>100</v>
+      </c>
+      <c r="E12" t="n">
+        <v>100</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G12" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B13" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C13" s="171" t="n">
+        <v>81</v>
+      </c>
+      <c r="D13" s="171" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" s="171" t="n">
+        <v>100</v>
+      </c>
+      <c r="F13" s="171" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G13" s="172" t="n">
+        <v>100</v>
+      </c>
+      <c r="H13" s="171" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B14" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C14" s="171" t="n">
+        <v>76</v>
+      </c>
+      <c r="D14" s="171" t="n">
+        <v>94</v>
+      </c>
+      <c r="E14" s="171" t="n">
+        <v>100</v>
+      </c>
+      <c r="F14" s="171" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G14" s="172" t="n">
+        <v>100</v>
+      </c>
+      <c r="H14" s="171" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>81</v>
+      </c>
+      <c r="D15" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" t="n">
+        <v>100</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G15" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>70</v>
+      </c>
+      <c r="D16" t="n">
+        <v>86</v>
+      </c>
+      <c r="E16" t="n">
+        <v>100</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G16" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>81</v>
+      </c>
+      <c r="D17" t="n">
+        <v>100</v>
+      </c>
+      <c r="E17" t="n">
+        <v>100</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="G17" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>70</v>
+      </c>
+      <c r="D18" t="n">
+        <v>86</v>
+      </c>
+      <c r="E18" t="n">
+        <v>100</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G18" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>100</v>
+      </c>
+      <c r="D19" t="n">
+        <v>100</v>
+      </c>
+      <c r="E19" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G19" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>73</v>
+      </c>
+      <c r="D20" t="n">
+        <v>91</v>
+      </c>
+      <c r="E20" t="n">
+        <v>100</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G20" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>70</v>
+      </c>
+      <c r="D21" t="n">
+        <v>86</v>
+      </c>
+      <c r="E21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G21" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>100</v>
+      </c>
+      <c r="D22" t="n">
+        <v>100</v>
+      </c>
+      <c r="E22" t="n">
+        <v>100</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G22" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>100</v>
+      </c>
+      <c r="D23" t="n">
+        <v>100</v>
+      </c>
+      <c r="E23" t="n">
+        <v>100</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="G23" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>76</v>
+      </c>
+      <c r="D24" t="n">
+        <v>94</v>
+      </c>
+      <c r="E24" t="n">
+        <v>100</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G24" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="166" t="inlineStr">
+        <is>
+          <t>INFERRED PRICE TIERS (cheapest first)</t>
+        </is>
+      </c>
+      <c r="B27" s="166" t="inlineStr">
+        <is>
+          <t>Rec</t>
+        </is>
+      </c>
+      <c r="C27" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="D27" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="E27" s="166" t="inlineStr">
+        <is>
+          <t>Brands at this price</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tier 100</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>100</v>
+      </c>
+      <c r="C28" t="n">
+        <v>100</v>
+      </c>
+      <c r="D28" t="n">
+        <v>100</v>
+      </c>
+      <c r="E28" s="170" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy (Spoke'd Up), Mars Rover (SpaceBikes), Whole MILC MKII (MILC Bikes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>tier 92</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>92</v>
+      </c>
+      <c r="C29" t="n">
+        <v>100</v>
+      </c>
+      <c r="D29" t="n">
+        <v>100</v>
+      </c>
+      <c r="E29" s="170" t="inlineStr">
+        <is>
+          <t>MountainCruise1 (Bike Bros)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tier 85</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>85</v>
+      </c>
+      <c r="C30" t="n">
+        <v>100</v>
+      </c>
+      <c r="D30" t="n">
+        <v>100</v>
+      </c>
+      <c r="E30" s="170" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro (LiteCycle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tier 83</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>83</v>
+      </c>
+      <c r="C31" t="n">
+        <v>100</v>
+      </c>
+      <c r="D31" t="n">
+        <v>100</v>
+      </c>
+      <c r="E31" s="170" t="inlineStr">
+        <is>
+          <t>LiteSpeed+ (LiteCycle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tier 82</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>82</v>
+      </c>
+      <c r="C32" t="n">
+        <v>100</v>
+      </c>
+      <c r="D32" t="n">
+        <v>100</v>
+      </c>
+      <c r="E32" s="170" t="inlineStr">
+        <is>
+          <t>TERRAMean (Bike Bros)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="173" t="inlineStr">
+        <is>
+          <t>tier 81</t>
+        </is>
+      </c>
+      <c r="B33" s="173" t="n">
+        <v>81</v>
+      </c>
+      <c r="C33" s="173" t="n">
+        <v>100</v>
+      </c>
+      <c r="D33" s="173" t="n">
+        <v>100</v>
+      </c>
+      <c r="E33" s="193" t="inlineStr">
+        <is>
+          <t>Hike Bike (WeBike), Blu Ruged Ballz (BB LLC), Blu Tail Ballz (BB LLC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="173" t="inlineStr">
+        <is>
+          <t>tier 76</t>
+        </is>
+      </c>
+      <c r="B34" s="173" t="n">
+        <v>76</v>
+      </c>
+      <c r="C34" s="173" t="n">
+        <v>94</v>
+      </c>
+      <c r="D34" s="173" t="n">
+        <v>100</v>
+      </c>
+      <c r="E34" s="193" t="inlineStr">
+        <is>
+          <t>Swift Bike (WeBike), Skim MILC MKII (MILC Bikes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>tier 73</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>73</v>
+      </c>
+      <c r="C35" t="n">
+        <v>91</v>
+      </c>
+      <c r="D35" t="n">
+        <v>100</v>
+      </c>
+      <c r="E35" s="170" t="inlineStr">
+        <is>
+          <t>TERRAMAX (Bike Bros), Spoke'd Speed (Spoke'd Up)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>tier 73</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>73</v>
+      </c>
+      <c r="C36" t="n">
+        <v>90</v>
+      </c>
+      <c r="D36" t="n">
+        <v>100</v>
+      </c>
+      <c r="E36" s="170" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+ (LiteCycle)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>tier 70</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>70</v>
+      </c>
+      <c r="C37" t="n">
+        <v>86</v>
+      </c>
+      <c r="D37" t="n">
+        <v>100</v>
+      </c>
+      <c r="E37" s="170" t="inlineStr">
+        <is>
+          <t>Mach 0.6 (Bike Bros), Blu Aero Ballz (BB LLC), Blu Tube Ballz (BB LLC), The Armstrong (SpaceBikes)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>tier 63</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>63</v>
+      </c>
+      <c r="C38" t="n">
+        <v>78</v>
+      </c>
+      <c r="D38" t="n">
+        <v>90</v>
+      </c>
+      <c r="E38" s="170" t="inlineStr">
+        <is>
+          <t>MACH I.I (Bike Bros)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="166" t="inlineStr">
+        <is>
+          <t>SEGMENT PRICE SENSITIVITY — resistance sets in at different tiers</t>
+        </is>
+      </c>
+      <c r="B41" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="C41" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="D41" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>tier 100 (cheapest)</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>100</v>
+      </c>
+      <c r="C42" t="n">
+        <v>100</v>
+      </c>
+      <c r="D42" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>tier 92</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>100</v>
+      </c>
+      <c r="C43" t="n">
+        <v>100</v>
+      </c>
+      <c r="D43" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>tier 85</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>100</v>
+      </c>
+      <c r="C44" t="n">
+        <v>100</v>
+      </c>
+      <c r="D44" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>tier 83</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>100</v>
+      </c>
+      <c r="C45" t="n">
+        <v>100</v>
+      </c>
+      <c r="D45" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>tier 82</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>100</v>
+      </c>
+      <c r="C46" t="n">
+        <v>100</v>
+      </c>
+      <c r="D46" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>tier 81  &lt;- Hike Bike</t>
+        </is>
+      </c>
+      <c r="B47" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="C47" t="n">
+        <v>100</v>
+      </c>
+      <c r="D47" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>tier 76  &lt;- Swift Bike</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>94</v>
+      </c>
+      <c r="C48" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="D48" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>tier 73</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>91</v>
+      </c>
+      <c r="C49" t="n">
+        <v>100</v>
+      </c>
+      <c r="D49" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>tier 70</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>86</v>
+      </c>
+      <c r="C50" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="D50" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>tier 63 (most expensive)</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>78</v>
+      </c>
+      <c r="C51" s="167" t="n">
+        <v>90</v>
+      </c>
+      <c r="D51" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D52" s="174" t="inlineStr">
+        <is>
+          <t>SPEED is the least price-sensitive segment in the game - it tolerates every price up to tier 70 with zero resistance. MOUNTAIN starts resisting immediately below tier 81. RECREATION resists almost everything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="166" t="inlineStr">
+        <is>
+          <t>HIKE BIKE — price is already optimal, hold it</t>
+        </is>
+      </c>
+      <c r="B55" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C55" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1365</v>
+      </c>
+      <c r="C56" s="170" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Mountain price judgment</t>
+        </is>
+      </c>
+      <c r="B57" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="C57" s="170" t="inlineStr">
+        <is>
+          <t>ZERO price resistance</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Price tier</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>81</v>
+      </c>
+      <c r="C58" s="170" t="inlineStr">
+        <is>
+          <t>the HIGHEST-priced tier that still scores 100 in Mountain</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Next tier up (73)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>91</v>
+      </c>
+      <c r="C59" s="170" t="inlineStr">
+        <is>
+          <t>TERRAMAX sits there and takes a 9-point hit</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="C60" s="181" t="inlineStr">
+        <is>
+          <t>We are extracting the maximum price Mountain will bear without penalty. Raising it drops us into the resistance band. HOLD $1,365.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="166" t="inlineStr">
+        <is>
+          <t>SWIFT BIKE — we are UNDER-priced in Speed</t>
+        </is>
+      </c>
+      <c r="B63" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C63" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C64" s="170" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Speed price judgment</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>100</v>
+      </c>
+      <c r="C65" s="170" t="inlineStr">
+        <is>
+          <t>zero resistance</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Our price tier</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>76</v>
+      </c>
+      <c r="C66" s="170" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Tier 70 brands (Armstrong, Blu Tube, Blu Aero, Mach 0.6)</t>
+        </is>
+      </c>
+      <c r="B67" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="C67" s="170" t="inlineStr">
+        <is>
+          <t>priced ABOVE us and STILL score 100 in Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>First tier with Speed resistance</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>63</v>
+      </c>
+      <c r="C68" s="170" t="inlineStr">
+        <is>
+          <t>only MACH I.I, at 90</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Headroom</t>
+        </is>
+      </c>
+      <c r="C69" s="170" t="inlineStr">
+        <is>
+          <t>roughly 1-2 price tiers before Speed resistance appears</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Estimated tier-70 price</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1595</v>
+      </c>
+      <c r="C70" s="170" t="inlineStr">
+        <is>
+          <t>INFERRED - see the estimate note below</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Potential price increase</t>
+        </is>
+      </c>
+      <c r="B71">
+        <f>C70-C64</f>
+        <v/>
+      </c>
+      <c r="C71" s="170" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>On Q3 volume (215 units)</t>
+        </is>
+      </c>
+      <c r="B72" s="159">
+        <f>C71*215</f>
+        <v/>
+      </c>
+      <c r="C72" s="170" t="inlineStr">
+        <is>
+          <t>pure margin - no cost change</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>On a rebuilt Speed volume (say 400 units)</t>
+        </is>
+      </c>
+      <c r="B73" s="159">
+        <f>C71*400</f>
+        <v/>
+      </c>
+      <c r="C73" s="170" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>CAVEAT</t>
+        </is>
+      </c>
+      <c r="C74" s="174" t="inlineStr">
+        <is>
+          <t>The $1,595 figure is inferred from BB LLC's ~$1,480 average price across 4 brands, two of which appear to sit at our $1,365 tier. VERIFY against the actual price list before locking. The DIRECTION (we have room to raise) is solid; the exact number is not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="166" t="inlineStr">
+        <is>
+          <t>THE BB LLC COMPARISON IS NOW AIRTIGHT</t>
+        </is>
+      </c>
+      <c r="B77" s="166" t="inlineStr">
+        <is>
+          <t>Hike Bike (WeBike)</t>
+        </is>
+      </c>
+      <c r="C77" s="166" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz (BB LLC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Brand judgment - Mountain</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>73</v>
+      </c>
+      <c r="C78" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Component recipe</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>56/73/1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>56/73/1 (identical)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Price judgment</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>81 / 100 / 100</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>81 / 100 / 100 (identical)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Implied price</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>$1,365</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>$1,365 (same tier)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Mountain share</t>
+        </is>
+      </c>
+      <c r="B82" s="179" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="C82" s="161" t="n">
+        <v>0.463</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Conclusion</t>
+        </is>
+      </c>
+      <c r="C83" s="174" t="inlineStr">
+        <is>
+          <t>Same product, same price, same price perception - and they take 2.1x our share. There is now no product or pricing explanation left. The entire gap is SUPPLY (we stocked out 33%), COVERAGE (14 store staff vs 14 but 7 web vs our 3) and ADS (24 regional vs our 19).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="166" t="inlineStr">
+        <is>
+          <t>ANOTHER REASON TO SKIP RECREATION</t>
+        </is>
+      </c>
+      <c r="B86" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C86" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Hike Bike Recreation price judgment</t>
+        </is>
+      </c>
+      <c r="B87" s="167" t="n">
+        <v>81</v>
+      </c>
+      <c r="C87" s="170" t="inlineStr">
+        <is>
+          <t>Rec buyers resist our $1,365</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>All three Recreation brands</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>100</v>
+      </c>
+      <c r="C88" s="170" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy, Mars Rover, Whole MILC - all at tier 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C89" s="170" t="inlineStr">
+        <is>
+          <t>Recreation is the most price-sensitive segment AND the winning brands are the cheapest in the game. Entering would mean a low-price, low-margin product - the opposite of our 'profit margin leader' strategy. Combined with the 56-vs-76 brand judgment gap, Recreation stays parked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="166" t="inlineStr">
+        <is>
+          <t>Q4 PRICING ACTIONS</t>
+        </is>
+      </c>
+      <c r="B92" s="166" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B93" s="174" t="inlineStr">
+        <is>
+          <t>HOLD $1,365. Mountain judgment 100 and we sit at the top tier that achieves it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B94" s="174" t="inlineStr">
+        <is>
+          <t>RAISE. Speed tolerates 1-2 tiers above us with zero resistance. Verify the exact price list, then move toward the Armstrong / Blu Tube tier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Sequencing note</t>
+        </is>
+      </c>
+      <c r="B95" s="174" t="inlineStr">
+        <is>
+          <t>Raise the Swift Bike price in the SAME quarter we fix its design to 77 - better product plus a price the segment does not resist is the cleanest margin gain available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Capacity note</t>
+        </is>
+      </c>
+      <c r="B96" s="174" t="inlineStr">
+        <is>
+          <t>A price rise also RELIEVES the capacity squeeze: more margin per unit on the same 24/day. If we cannot build 1,171 units, we should at least earn more on the ones we do build.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Q3 price list and confirm the inferred tiers.
Actual net prices rise monotonically across all ten inferred tiers and identical
price judgment meant identical price every time, putting the tier-70 estimate
within 15 dollars. Swift Bike can move to 1,580 with no Speed resistance, which
makes it our highest-contribution unit just as capacity becomes binding.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -42,6 +42,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Staffing" sheetId="34" state="visible" r:id="rId34"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Web_Ops" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Price_Judgment" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Prices" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -626,7 +627,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="195">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -899,6 +900,9 @@
     <xf numFmtId="165" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="30" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -34479,6 +34483,1947 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J100"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" style="146" min="1" max="1"/>
+    <col width="24" customWidth="1" style="146" min="2" max="2"/>
+    <col width="26" customWidth="1" style="146" min="3" max="3"/>
+    <col width="62" customWidth="1" style="146" min="4" max="4"/>
+    <col width="34" customWidth="1" style="146" min="5" max="5"/>
+    <col width="14" customWidth="1" style="146" min="6" max="6"/>
+    <col width="14" customWidth="1" style="146" min="7" max="7"/>
+    <col width="14" customWidth="1" style="146" min="8" max="8"/>
+    <col width="14" customWidth="1" style="146" min="9" max="9"/>
+    <col width="14" customWidth="1" style="146" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Competitors' Prices — World Market, Q3 actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>Actual price list. It confirms the price tiers inferred from price judgment: every tier maps to a distinct price, monotonically, across all 11 tiers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Rebate</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Net price</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>Brand judgment</t>
+        </is>
+      </c>
+      <c r="I4" s="166" t="inlineStr">
+        <is>
+          <t>Price judgment</t>
+        </is>
+      </c>
+      <c r="J4" s="166" t="inlineStr">
+        <is>
+          <t>Price tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1749</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1749</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>77</v>
+      </c>
+      <c r="I5" s="167" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1580</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1580</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>74</v>
+      </c>
+      <c r="I6" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1580</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1580</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>76</v>
+      </c>
+      <c r="I7" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1580</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1580</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>76</v>
+      </c>
+      <c r="I8" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mach 0.6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1579</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1579</v>
+      </c>
+      <c r="F9" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>61</v>
+      </c>
+      <c r="I9" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1515</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1515</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>77</v>
+      </c>
+      <c r="I10" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1499</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>73</v>
+      </c>
+      <c r="I11" s="167" t="n">
+        <v>91</v>
+      </c>
+      <c r="J11" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1499</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1499</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>75</v>
+      </c>
+      <c r="I12" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J12" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B13" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C13" s="171" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D13" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="171" t="n">
+        <v>1450</v>
+      </c>
+      <c r="F13" s="171" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="171" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H13" s="171" t="n">
+        <v>72</v>
+      </c>
+      <c r="I13" s="172" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" s="171" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>1450</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1450</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>76</v>
+      </c>
+      <c r="I14" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J14" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B15" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C15" s="171" t="n">
+        <v>1365</v>
+      </c>
+      <c r="D15" s="171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="171" t="n">
+        <v>1365</v>
+      </c>
+      <c r="F15" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="171" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H15" s="171" t="n">
+        <v>73</v>
+      </c>
+      <c r="I15" s="172" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" s="171" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1365</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1365</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>73</v>
+      </c>
+      <c r="I16" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J16" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1365</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1365</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>70</v>
+      </c>
+      <c r="I17" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TERRAMean</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1349</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1349</v>
+      </c>
+      <c r="F18" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>72</v>
+      </c>
+      <c r="I18" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J18" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1325</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1325</v>
+      </c>
+      <c r="F19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>74</v>
+      </c>
+      <c r="I19" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1300</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1300</v>
+      </c>
+      <c r="F20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>70</v>
+      </c>
+      <c r="I20" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>MountainCruise1</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1199</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1199</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>76</v>
+      </c>
+      <c r="I21" s="167" t="n">
+        <v>92</v>
+      </c>
+      <c r="J21" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1100</v>
+      </c>
+      <c r="D22" t="n">
+        <v>50</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1050</v>
+      </c>
+      <c r="F22" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>73</v>
+      </c>
+      <c r="I22" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>999</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>999</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>73</v>
+      </c>
+      <c r="I23" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1050</v>
+      </c>
+      <c r="D24" t="n">
+        <v>100</v>
+      </c>
+      <c r="E24" t="n">
+        <v>950</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>74</v>
+      </c>
+      <c r="I24" s="159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J24" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="166" t="inlineStr">
+        <is>
+          <t>TIER VALIDATION — inferred tier vs actual net price</t>
+        </is>
+      </c>
+      <c r="B27" s="166" t="inlineStr">
+        <is>
+          <t>Net price range</t>
+        </is>
+      </c>
+      <c r="C27" s="166" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="D27" s="166" t="inlineStr">
+        <is>
+          <t>Brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tier 100</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>950 - 1,050</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>100</v>
+      </c>
+      <c r="D28" s="170" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy, Mars Rover, Whole MILC MKII</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>tier 92</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1,199 - 1,199</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="170" t="inlineStr">
+        <is>
+          <t>MountainCruise1</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>tier 85</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1,300 - 1,300</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="170" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tier 83</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1,325 - 1,325</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="170" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>tier 82</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1,349 - 1,349</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="170" t="inlineStr">
+        <is>
+          <t>TERRAMean</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>tier 81</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1,365 - 1,365</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="170" t="inlineStr">
+        <is>
+          <t>Hike Bike, Blu Ruged Ballz, Blu Tail Ballz</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>tier 76</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1,450 - 1,450</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="170" t="inlineStr">
+        <is>
+          <t>Swift Bike, Skim MILC MKII</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>tier 73</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1,499 - 1,515</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>16</v>
+      </c>
+      <c r="D35" s="170" t="inlineStr">
+        <is>
+          <t>TERRAMAX, LiteSpeed Pro+, Spoke'd Speed</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>tier 70</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1,579 - 1,580</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="170" t="inlineStr">
+        <is>
+          <t>Mach 0.6, Blu Aero Ballz, Blu Tube Ballz, The Armstrong</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>tier 63</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1,749 - 1,749</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="170" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="D38" s="181" t="inlineStr">
+        <is>
+          <t>Perfectly monotonic. Identical price judgment DID mean identical price in every case. Our earlier $1,595 estimate for tier 70 came in at $1,580 - off by $15 (0.9%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="166" t="inlineStr">
+        <is>
+          <t>SPEED PRICE LADDER — we are nearly the cheapest</t>
+        </is>
+      </c>
+      <c r="B41" s="166" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C41" s="166" t="inlineStr">
+        <is>
+          <t>Brand judgment</t>
+        </is>
+      </c>
+      <c r="D41" s="166" t="inlineStr">
+        <is>
+          <t>Price judgment</t>
+        </is>
+      </c>
+      <c r="E41" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C42" t="n">
+        <v>77</v>
+      </c>
+      <c r="D42" t="n">
+        <v>90</v>
+      </c>
+      <c r="E42" s="170" t="inlineStr">
+        <is>
+          <t>only Speed brand with price resistance</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Blu Aero Ballz</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C43" t="n">
+        <v>74</v>
+      </c>
+      <c r="D43" t="n">
+        <v>100</v>
+      </c>
+      <c r="E43" s="170" t="inlineStr">
+        <is>
+          <t>highest price with ZERO resistance</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C44" t="n">
+        <v>76</v>
+      </c>
+      <c r="D44" t="n">
+        <v>100</v>
+      </c>
+      <c r="E44" s="170" t="inlineStr">
+        <is>
+          <t>highest price with ZERO resistance</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C45" t="n">
+        <v>76</v>
+      </c>
+      <c r="D45" t="n">
+        <v>100</v>
+      </c>
+      <c r="E45" s="170" t="inlineStr">
+        <is>
+          <t>highest price with ZERO resistance</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Mach 0.6</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1579</v>
+      </c>
+      <c r="C46" t="n">
+        <v>61</v>
+      </c>
+      <c r="D46" t="n">
+        <v>100</v>
+      </c>
+      <c r="E46" s="170" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1515</v>
+      </c>
+      <c r="C47" t="n">
+        <v>77</v>
+      </c>
+      <c r="D47" t="n">
+        <v>100</v>
+      </c>
+      <c r="E47" s="170" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1499</v>
+      </c>
+      <c r="C48" t="n">
+        <v>75</v>
+      </c>
+      <c r="D48" t="n">
+        <v>100</v>
+      </c>
+      <c r="E48" s="170" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B49" s="171" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C49" s="171" t="n">
+        <v>72</v>
+      </c>
+      <c r="D49" s="171" t="n">
+        <v>100</v>
+      </c>
+      <c r="E49" s="194" t="inlineStr">
+        <is>
+          <t>OURS - 2nd cheapest, 2nd worst product</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C50" t="n">
+        <v>76</v>
+      </c>
+      <c r="D50" t="n">
+        <v>100</v>
+      </c>
+      <c r="E50" s="170" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C51" t="n">
+        <v>74</v>
+      </c>
+      <c r="D51" t="n">
+        <v>100</v>
+      </c>
+      <c r="E51" s="170" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="166" t="inlineStr">
+        <is>
+          <t>SWIFT BIKE PRICE MOVE — now precise</t>
+        </is>
+      </c>
+      <c r="B54" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C54" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Current price</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C55" s="170" t="inlineStr">
+        <is>
+          <t>2nd cheapest of 10 Speed brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Speed median price</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>1547</v>
+      </c>
+      <c r="C56" s="170" t="inlineStr">
+        <is>
+          <t>we sit $97 below the median</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Highest price with ZERO Speed resistance</t>
+        </is>
+      </c>
+      <c r="B57" s="159" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C57" s="170" t="inlineStr">
+        <is>
+          <t>Mach 0.6, Blu Aero, Blu Tube, The Armstrong</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>First price WITH resistance</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1749</v>
+      </c>
+      <c r="C58" s="170" t="inlineStr">
+        <is>
+          <t>MACH I.I, judgment 90</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Safe increase</t>
+        </is>
+      </c>
+      <c r="B59" s="159">
+        <f>C57-C55</f>
+        <v/>
+      </c>
+      <c r="C59" s="170" t="inlineStr">
+        <is>
+          <t>proven safe by four rival brands</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>On Q3 volume (215 units)</t>
+        </is>
+      </c>
+      <c r="B60" s="159">
+        <f>C59*215</f>
+        <v/>
+      </c>
+      <c r="C60" s="170" t="inlineStr">
+        <is>
+          <t>pure margin, no cost change</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>On a rebuilt Speed volume (400 units)</t>
+        </is>
+      </c>
+      <c r="B61" s="159">
+        <f>C59*400</f>
+        <v/>
+      </c>
+      <c r="C61" s="170" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Untested zone</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>1,581 - 1,748</t>
+        </is>
+      </c>
+      <c r="C62" s="170" t="inlineStr">
+        <is>
+          <t>nobody prices here, so resistance onset is unknown. $1,580 is the evidence-backed target.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="166" t="inlineStr">
+        <is>
+          <t>HIKE BIKE — confirmed at the Mountain ceiling</t>
+        </is>
+      </c>
+      <c r="B65" s="166" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C65" s="166" t="inlineStr">
+        <is>
+          <t>Mountain price judgment</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1300</v>
+      </c>
+      <c r="C66" s="170" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>LiteSpeed+ (Speed brand)</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1325</v>
+      </c>
+      <c r="C67" s="170" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>TERRAMean</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1349</v>
+      </c>
+      <c r="C68" s="170" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Hike Bike / Blu Ruged Ballz / Blu Tail Ballz</t>
+        </is>
+      </c>
+      <c r="B69" s="159" t="n">
+        <v>1365</v>
+      </c>
+      <c r="C69" s="181" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Swift Bike / Skim MILC (tier above)</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C70" s="185" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1499</v>
+      </c>
+      <c r="C71" s="170" t="n">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="C72" s="170" t="inlineStr">
+        <is>
+          <t>Mountain resistance begins somewhere between $1,365 and $1,450. We sit at the top of the clean band. HOLD $1,365 - the $85 of untested space is not worth risking a judgment drop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="166" t="inlineStr">
+        <is>
+          <t>CONTRIBUTION PER UNIT — matters now that capacity binds</t>
+        </is>
+      </c>
+      <c r="B75" s="166" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C75" s="166" t="inlineStr">
+        <is>
+          <t>Q3 unit cost</t>
+        </is>
+      </c>
+      <c r="D75" s="166" t="inlineStr">
+        <is>
+          <t>Contribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1365</v>
+      </c>
+      <c r="C76" t="n">
+        <v>618</v>
+      </c>
+      <c r="D76" s="170">
+        <f>B76-C76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Swift Bike (today)</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1450</v>
+      </c>
+      <c r="C77" t="n">
+        <v>694</v>
+      </c>
+      <c r="D77" s="170">
+        <f>B77-C77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Swift Bike at $1,580</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C78" t="n">
+        <v>694</v>
+      </c>
+      <c r="D78" s="181">
+        <f>B78-C78</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Swift Bike at $1,580 with 14-speed gears</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1580</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>lower</t>
+        </is>
+      </c>
+      <c r="D79" s="170" t="inlineStr">
+        <is>
+          <t>higher still</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D80" s="174" t="inlineStr">
+        <is>
+          <t>At $1,580 Swift Bike becomes our MOST profitable unit ($886 vs Hike Bike's $747). Switching it to 14-speed (the design fix) should cut its cost too, widening the gap further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="166" t="inlineStr">
+        <is>
+          <t>PRIORITY FIELD — a lever we have not thought about</t>
+        </is>
+      </c>
+      <c r="B83" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C83" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Our priority order</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1 Hike Bike, 2 Swift Bike</t>
+        </is>
+      </c>
+      <c r="C84" s="170" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Q3 stock-out by brand</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Hike Bike 134/412 = 32.5%</t>
+        </is>
+      </c>
+      <c r="C85" s="170" t="inlineStr">
+        <is>
+          <t>Swift Bike 70/215 = 32.6%</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="C86" s="170" t="inlineStr">
+        <is>
+          <t>Both brands lost almost exactly the same percentage, so priority 1 did NOT shield Hike Bike in Q3. Treat the mechanism as unverified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Why it matters in Q4</t>
+        </is>
+      </c>
+      <c r="C87" s="174" t="inlineStr">
+        <is>
+          <t>Capacity is now binding (see Q4_Planner). If we cannot build all demand, the priority order decides the mix. After the price rise, Swift Bike earns $886/unit vs Hike Bike's $747 - so a pure margin view argues for promoting Swift Bike.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Counter-argument</t>
+        </is>
+      </c>
+      <c r="C88" s="174" t="inlineStr">
+        <is>
+          <t>Mountain is our PRIMARY segment for the Balanced Scorecard's Market Performance, and we hold 22.1% there vs 7.5% in Speed. Starving Hike Bike would hurt the scorecard even if it helps the income statement. Decide deliberately - do not leave it on default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Rebates</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>we use 0</t>
+        </is>
+      </c>
+      <c r="C89" s="170" t="inlineStr">
+        <is>
+          <t>Only the two Recreation leaders rebate: Mars Rover $50, Whole MILC $100. Rebates appear to be a Recreation/price-sensitive tool - no reason for us to start.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="166" t="inlineStr">
+        <is>
+          <t>HOW RIVALS PRICE BY SEGMENT — the pattern to copy</t>
+        </is>
+      </c>
+      <c r="B92" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="C92" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="D92" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>$1,365</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>$1,580</t>
+        </is>
+      </c>
+      <c r="D93" s="170" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>$1,580</t>
+        </is>
+      </c>
+      <c r="D94" s="170" t="inlineStr">
+        <is>
+          <t>$1,050 net</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>$1,450</t>
+        </is>
+      </c>
+      <c r="D95" s="170" t="inlineStr">
+        <is>
+          <t>$950 net</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>$1,300</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>$1,325 - $1,515</t>
+        </is>
+      </c>
+      <c r="D96" s="170" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>$1,349 - $1,499</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>$1,579 - $1,749</t>
+        </is>
+      </c>
+      <c r="D97" s="170" t="inlineStr">
+        <is>
+          <t>$1,199</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>$1,499</t>
+        </is>
+      </c>
+      <c r="D98" s="170" t="inlineStr">
+        <is>
+          <t>$999</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B99" s="171" t="inlineStr">
+        <is>
+          <t>$1,365</t>
+        </is>
+      </c>
+      <c r="C99" s="171" t="inlineStr">
+        <is>
+          <t>$1,450</t>
+        </is>
+      </c>
+      <c r="D99" s="194" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D100" s="174" t="inlineStr">
+        <is>
+          <t>The strong firms price Speed $200+ above Mountain and Recreation far below. BB LLC is the cleanest example: identical Mountain price to ours, Speed $215 higher. We copied their Mountain price correctly and missed their Speed price entirely.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add Q3 ad judgment and confirm the Marketing Effectiveness formula
Ad judgment was the missing input, and the class formula now reproduces all
three reported figures exactly: our 0.738, BB LLC's 0.765 industry max, and
Spoke'd Up's 0.660 minimum. That turns the Swift Bike question into arithmetic.

HikeBike 1 scores 80 in Mountain, one point off the industry best, so it stays
as is. The Swift Bike ad is 8th of 9 in Speed at 70 while leaking 88 points into
Recreation and Mountain against 12-46 for every rival, which looks like the same
mistake as the 24-speed drivetrain: Hike Bike's playbook cloned into a Speed
launch. Fixing the brand and the ad together lifts Marketing Effectiveness to
0.7675, past BB LLC, on an indicator where we sit below average today.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/quarters/Q3/Q3Data.xlsx
+++ b/quarters/Q3/Q3Data.xlsx
@@ -43,6 +43,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Web_Ops" sheetId="35" state="visible" r:id="rId35"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Price_Judgment" sheetId="36" state="visible" r:id="rId36"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Prices" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_Ad_Judgment" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -51,9 +52,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
   <fonts count="31">
     <font>
@@ -627,7 +629,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="16"/>
   </cellStyleXfs>
-  <cellXfs count="195">
+  <cellXfs count="199">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -905,6 +907,10 @@
     <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="28" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="28" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -36424,6 +36430,1558 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I84"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" style="146" min="1" max="1"/>
+    <col width="22" customWidth="1" style="146" min="2" max="2"/>
+    <col width="22" customWidth="1" style="146" min="3" max="3"/>
+    <col width="62" customWidth="1" style="146" min="4" max="4"/>
+    <col width="40" customWidth="1" style="146" min="5" max="5"/>
+    <col width="15" customWidth="1" style="146" min="6" max="6"/>
+    <col width="15" customWidth="1" style="146" min="7" max="7"/>
+    <col width="15" customWidth="1" style="146" min="8" max="8"/>
+    <col width="15" customWidth="1" style="146" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="169" t="inlineStr">
+        <is>
+          <t>Ad Judgment — World Market, Q3 actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="170" t="inlineStr">
+        <is>
+          <t>HikeBike 1 is essentially best-in-class (80 vs BB LLC's 81). The Swift Bike ad is 8th of 9 Speed ads and shows by far the highest off-target appeal in the industry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="166" t="inlineStr">
+        <is>
+          <t>Ad</t>
+        </is>
+      </c>
+      <c r="B4" s="166" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C4" s="166" t="inlineStr">
+        <is>
+          <t>Brand advertised</t>
+        </is>
+      </c>
+      <c r="D4" s="166" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="E4" s="166" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="F4" s="166" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="G4" s="166" t="inlineStr">
+        <is>
+          <t>Target segment</t>
+        </is>
+      </c>
+      <c r="H4" s="166" t="inlineStr">
+        <is>
+          <t>Score in target</t>
+        </is>
+      </c>
+      <c r="I4" s="166" t="inlineStr">
+        <is>
+          <t>Off-target leakage</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Excluspeedity</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F5" t="n">
+        <v>72</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>72</v>
+      </c>
+      <c r="I5" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TerraTech</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>23</v>
+      </c>
+      <c r="E6" t="n">
+        <v>78</v>
+      </c>
+      <c r="F6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>78</v>
+      </c>
+      <c r="I6" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Easy Rider</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MountainCruise1</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>75</v>
+      </c>
+      <c r="E7" t="n">
+        <v>25</v>
+      </c>
+      <c r="F7" t="n">
+        <v>17</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>75</v>
+      </c>
+      <c r="I7" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mountainability</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TERRAMAX</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>35</v>
+      </c>
+      <c r="E8" t="n">
+        <v>77</v>
+      </c>
+      <c r="F8" t="n">
+        <v>32</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>77</v>
+      </c>
+      <c r="I8" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AndStill</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MACH I.I</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>22</v>
+      </c>
+      <c r="E9" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" t="n">
+        <v>78</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>78</v>
+      </c>
+      <c r="I9" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Speed of Lite 1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>LiteSpeed Pro+</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="n">
+        <v>22</v>
+      </c>
+      <c r="F10" t="n">
+        <v>77</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>77</v>
+      </c>
+      <c r="I10" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Speed of Lite 2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LiteSpeed+</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>16</v>
+      </c>
+      <c r="E11" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" t="n">
+        <v>73</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>73</v>
+      </c>
+      <c r="I11" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Trail Blazing 1</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>LiteTrail Pro</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" t="n">
+        <v>79</v>
+      </c>
+      <c r="F12" t="n">
+        <v>34</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>79</v>
+      </c>
+      <c r="I12" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="171" t="inlineStr">
+        <is>
+          <t>HikeBike 1</t>
+        </is>
+      </c>
+      <c r="B13" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C13" s="171" t="inlineStr">
+        <is>
+          <t>Hike Bike</t>
+        </is>
+      </c>
+      <c r="D13" s="171" t="n">
+        <v>33</v>
+      </c>
+      <c r="E13" s="171" t="n">
+        <v>80</v>
+      </c>
+      <c r="F13" s="171" t="n">
+        <v>26</v>
+      </c>
+      <c r="G13" s="171" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H13" s="171" t="n">
+        <v>80</v>
+      </c>
+      <c r="I13" s="171" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="B14" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="C14" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike</t>
+        </is>
+      </c>
+      <c r="D14" s="171" t="n">
+        <v>52</v>
+      </c>
+      <c r="E14" s="171" t="n">
+        <v>36</v>
+      </c>
+      <c r="F14" s="171" t="n">
+        <v>70</v>
+      </c>
+      <c r="G14" s="171" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H14" s="171" t="n">
+        <v>70</v>
+      </c>
+      <c r="I14" s="171" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BB Big Momma</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Blu Ruged Ballz</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>28</v>
+      </c>
+      <c r="E15" t="n">
+        <v>81</v>
+      </c>
+      <c r="F15" t="n">
+        <v>27</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Mountain</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>81</v>
+      </c>
+      <c r="I15" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Unleash lil pap</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Blu Tube Ballz</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" t="n">
+        <v>16</v>
+      </c>
+      <c r="F16" t="n">
+        <v>76</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>76</v>
+      </c>
+      <c r="I16" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Spoke'd Easy</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>59</v>
+      </c>
+      <c r="E17" t="n">
+        <v>27</v>
+      </c>
+      <c r="F17" t="n">
+        <v>21</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>59</v>
+      </c>
+      <c r="I17" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" t="n">
+        <v>18</v>
+      </c>
+      <c r="F18" t="n">
+        <v>57</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>57</v>
+      </c>
+      <c r="I18" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>The Armstrong 1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>The Armstrong</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="n">
+        <v>21</v>
+      </c>
+      <c r="F19" t="n">
+        <v>77</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>77</v>
+      </c>
+      <c r="I19" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Mars Rover 1</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mars Rover</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>79</v>
+      </c>
+      <c r="E20" t="n">
+        <v>25</v>
+      </c>
+      <c r="F20" t="n">
+        <v>24</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>79</v>
+      </c>
+      <c r="I20" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>10</v>
+      </c>
+      <c r="E21" t="n">
+        <v>19</v>
+      </c>
+      <c r="F21" t="n">
+        <v>75</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Speed</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>75</v>
+      </c>
+      <c r="I21" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Whole MILC MKII</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>77</v>
+      </c>
+      <c r="E22" t="n">
+        <v>47</v>
+      </c>
+      <c r="F22" t="n">
+        <v>41</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Recreation</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>77</v>
+      </c>
+      <c r="I22" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="166" t="inlineStr">
+        <is>
+          <t>SPEED AD LADDER</t>
+        </is>
+      </c>
+      <c r="B25" s="166" t="inlineStr">
+        <is>
+          <t>Speed score</t>
+        </is>
+      </c>
+      <c r="C25" s="166" t="inlineStr">
+        <is>
+          <t>Off-target leakage</t>
+        </is>
+      </c>
+      <c r="D25" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AndStill (Bike Bros)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>78</v>
+      </c>
+      <c r="C26" t="n">
+        <v>46</v>
+      </c>
+      <c r="D26" s="170" t="inlineStr">
+        <is>
+          <t>BEST Speed ad in the industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Speed of Lite 1 (LiteCycle)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>77</v>
+      </c>
+      <c r="C27" t="n">
+        <v>32</v>
+      </c>
+      <c r="D27" s="170" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>The Armstrong 1 (SpaceBikes)</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>77</v>
+      </c>
+      <c r="C28" t="n">
+        <v>23</v>
+      </c>
+      <c r="D28" s="170" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Unleash lil pap (BB LLC)</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>76</v>
+      </c>
+      <c r="C29" t="n">
+        <v>31</v>
+      </c>
+      <c r="D29" s="170" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Skim MILC MKII (MILC Bikes)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>75</v>
+      </c>
+      <c r="C30" t="n">
+        <v>29</v>
+      </c>
+      <c r="D30" s="170" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Speed of Lite 2 (LiteCycle)</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>73</v>
+      </c>
+      <c r="C31" t="n">
+        <v>29</v>
+      </c>
+      <c r="D31" s="170" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Excluspeedity (Bike Bros)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>72</v>
+      </c>
+      <c r="C32" t="n">
+        <v>12</v>
+      </c>
+      <c r="D32" s="170" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="171" t="inlineStr">
+        <is>
+          <t>Swift Bike (WeBike)</t>
+        </is>
+      </c>
+      <c r="B33" s="188" t="n">
+        <v>70</v>
+      </c>
+      <c r="C33" s="188" t="n">
+        <v>88</v>
+      </c>
+      <c r="D33" s="194" t="inlineStr">
+        <is>
+          <t>OURS - 8th of 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Spoke'd Speed (Spoke'd Up)</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>57</v>
+      </c>
+      <c r="C34" t="n">
+        <v>22</v>
+      </c>
+      <c r="D34" s="170" t="inlineStr">
+        <is>
+          <t>worst; drags Spoke'd Up to last on Marketing Effectiveness</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="166" t="inlineStr">
+        <is>
+          <t>MOUNTAIN AD LADDER</t>
+        </is>
+      </c>
+      <c r="B37" s="166" t="inlineStr">
+        <is>
+          <t>Mountain score</t>
+        </is>
+      </c>
+      <c r="C37" s="166" t="inlineStr">
+        <is>
+          <t>Off-target leakage</t>
+        </is>
+      </c>
+      <c r="D37" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BB Big Momma (BB LLC)</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>81</v>
+      </c>
+      <c r="C38" t="n">
+        <v>55</v>
+      </c>
+      <c r="D38" s="170" t="inlineStr">
+        <is>
+          <t>BEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="171" t="inlineStr">
+        <is>
+          <t>HikeBike 1 (WeBike)</t>
+        </is>
+      </c>
+      <c r="B39" s="172" t="n">
+        <v>80</v>
+      </c>
+      <c r="C39" s="171" t="n">
+        <v>59</v>
+      </c>
+      <c r="D39" s="194" t="inlineStr">
+        <is>
+          <t>OURS - 1 point off best</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Trail Blazing 1 (LiteCycle)</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>79</v>
+      </c>
+      <c r="C40" t="n">
+        <v>52</v>
+      </c>
+      <c r="D40" s="170" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>TerraTech (Bike Bros)</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>78</v>
+      </c>
+      <c r="C41" t="n">
+        <v>53</v>
+      </c>
+      <c r="D41" s="170" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Mountainability (Bike Bros)</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>77</v>
+      </c>
+      <c r="C42" t="n">
+        <v>67</v>
+      </c>
+      <c r="D42" s="170" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="166" t="inlineStr">
+        <is>
+          <t>MARKETING EFFECTIVENESS — formula verified against 3 reported values</t>
+        </is>
+      </c>
+      <c r="B45" s="166" t="inlineStr">
+        <is>
+          <t>Avg brand</t>
+        </is>
+      </c>
+      <c r="C45" s="166" t="inlineStr">
+        <is>
+          <t>Avg ad</t>
+        </is>
+      </c>
+      <c r="D45" s="166" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="E45" s="166" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="C46" t="n">
+        <v>78.5</v>
+      </c>
+      <c r="D46" s="195" t="n">
+        <v>0.765</v>
+      </c>
+      <c r="E46" s="170" t="n">
+        <v>0.765</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SpaceBikes</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="C47" t="n">
+        <v>78</v>
+      </c>
+      <c r="D47" s="195" t="n">
+        <v>0.7625</v>
+      </c>
+      <c r="E47" s="170" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>MILC Bikes</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>75</v>
+      </c>
+      <c r="C48" t="n">
+        <v>76</v>
+      </c>
+      <c r="D48" s="195" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="E48" s="170" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="171" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B49" s="171" t="n">
+        <v>72.5</v>
+      </c>
+      <c r="C49" s="171" t="n">
+        <v>75</v>
+      </c>
+      <c r="D49" s="196" t="n">
+        <v>0.7375</v>
+      </c>
+      <c r="E49" s="194" t="n">
+        <v>0.738</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>74</v>
+      </c>
+      <c r="C50" t="n">
+        <v>58</v>
+      </c>
+      <c r="D50" s="195" t="n">
+        <v>0.6599999999999999</v>
+      </c>
+      <c r="E50" s="170" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="E51" s="181" t="inlineStr">
+        <is>
+          <t>Industry min 0.660 (Spoke'd Up) and max 0.765 (BB LLC) both reproduce exactly, as does our 0.738. Formula confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="166" t="inlineStr">
+        <is>
+          <t>FIXING SWIFT BIKE — the Marketing Effectiveness payoff</t>
+        </is>
+      </c>
+      <c r="B54" s="166" t="inlineStr">
+        <is>
+          <t>Brand judgment</t>
+        </is>
+      </c>
+      <c r="C54" s="166" t="inlineStr">
+        <is>
+          <t>Ad judgment</t>
+        </is>
+      </c>
+      <c r="D54" s="166" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="E54" s="166" t="inlineStr">
+        <is>
+          <t>vs industry max 0.765</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Q3 actual</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>72</v>
+      </c>
+      <c r="C55" t="n">
+        <v>70</v>
+      </c>
+      <c r="D55" s="197" t="n">
+        <v>0.7375</v>
+      </c>
+      <c r="E55" s="170" t="inlineStr">
+        <is>
+          <t>below average (0.743)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Fix ad only</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>72</v>
+      </c>
+      <c r="C56" t="n">
+        <v>77</v>
+      </c>
+      <c r="D56" s="195" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="E56" s="170" t="inlineStr">
+        <is>
+          <t>3rd best</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Fix brand only (14-speed + decals)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>77</v>
+      </c>
+      <c r="C57" t="n">
+        <v>70</v>
+      </c>
+      <c r="D57" s="195" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E57" s="170" t="inlineStr">
+        <is>
+          <t>4th best</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>FIX BOTH</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>77</v>
+      </c>
+      <c r="C58" t="n">
+        <v>77</v>
+      </c>
+      <c r="D58" s="198" t="n">
+        <v>0.7675</v>
+      </c>
+      <c r="E58" s="181" t="inlineStr">
+        <is>
+          <t>NEW INDUSTRY BEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="166" t="inlineStr">
+        <is>
+          <t>DIAGNOSIS — the Swift Bike ad is unfocused</t>
+        </is>
+      </c>
+      <c r="B61" s="166" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C61" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Our Swift Bike ad: Recreation score</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>52</v>
+      </c>
+      <c r="C62" s="170" t="inlineStr">
+        <is>
+          <t>highest Rec score of ANY Speed ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Our Swift Bike ad: Mountain score</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>36</v>
+      </c>
+      <c r="C63" s="170" t="inlineStr">
+        <is>
+          <t>highest Mtn score of ANY Speed ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Total off-target leakage</t>
+        </is>
+      </c>
+      <c r="B64" s="167" t="n">
+        <v>88</v>
+      </c>
+      <c r="C64" s="170" t="inlineStr">
+        <is>
+          <t>next highest is AndStill at 46; The Armstrong 1 is just 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Leading Speed ads for comparison</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Rec 2-22, Mtn 13-24</t>
+        </is>
+      </c>
+      <c r="C65" s="170" t="inlineStr">
+        <is>
+          <t>The Armstrong 1 scores Rec 2 - almost zero</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Hypothesis</t>
+        </is>
+      </c>
+      <c r="C66" s="174" t="inlineStr">
+        <is>
+          <t>The ad appears to carry Mountain- and Recreation-flavoured benefit claims rather than Speed-specific ones. This MIRRORS the component error: Swift Bike inherited Hike Bike's 24-speed drivetrain AND, it seems, Hike Bike's messaging. Same root cause - we cloned our Mountain assets into a Speed launch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>CAUTION</t>
+        </is>
+      </c>
+      <c r="C67" s="174" t="inlineStr">
+        <is>
+          <t>Leakage does NOT cleanly predict score across the field (AndStill leaks 46 and scores best), so this is a strong hypothesis, not a solved model like the component analysis. Rebuild the ad around Speed cues and re-test in the ad designer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="166" t="inlineStr">
+        <is>
+          <t>AD PORTFOLIO PATTERNS</t>
+        </is>
+      </c>
+      <c r="B70" s="166" t="inlineStr">
+        <is>
+          <t>Ads</t>
+        </is>
+      </c>
+      <c r="C70" s="166" t="inlineStr">
+        <is>
+          <t>Brands</t>
+        </is>
+      </c>
+      <c r="D70" s="166" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Bike Bros</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>5</v>
+      </c>
+      <c r="C71" t="n">
+        <v>5</v>
+      </c>
+      <c r="D71" s="170" t="inlineStr">
+        <is>
+          <t>TWO ads each for MACH I.I and TERRAMAX - A/B testing. Still finished LAST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>LiteCycle</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n">
+        <v>3</v>
+      </c>
+      <c r="D72" s="170" t="inlineStr">
+        <is>
+          <t>one ad per brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>BB LLC</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2</v>
+      </c>
+      <c r="C73" t="n">
+        <v>4</v>
+      </c>
+      <c r="D73" s="170" t="inlineStr">
+        <is>
+          <t>advertises only Blu Ruged Ballz + Blu Tube Ballz; Blu Aero and Blu Tail run with NO ad</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>WeBike</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>2</v>
+      </c>
+      <c r="C74" t="n">
+        <v>2</v>
+      </c>
+      <c r="D74" s="170" t="inlineStr">
+        <is>
+          <t>one per brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>SpaceBikes / MILC / Spoke'd Up</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" t="n">
+        <v>2</v>
+      </c>
+      <c r="D75" s="170" t="inlineStr">
+        <is>
+          <t>one per brand</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="D76" s="174" t="inlineStr">
+        <is>
+          <t>The LEADER runs the FEWEST ads relative to its brand count - 2 ads for 4 brands - and both are best or near-best in class. Bike Bros runs the most ads and is last. Ad QUALITY beats ad COUNT. A second Swift Bike ad is not the answer; a better one is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Portfolio idea worth noting</t>
+        </is>
+      </c>
+      <c r="D77" s="170" t="inlineStr">
+        <is>
+          <t>BB LLC pairs an ADVERTISED brand with an UNADVERTISED second brand in each segment (Blu Ruged + Blu Tail in Mountain, Blu Tube + Blu Aero in Speed). The ad builds the segment and the second brand catches overflow at a higher price. Not a Q4 move for us - capacity binds - but note it for later.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="166" t="inlineStr">
+        <is>
+          <t>Q4 ADVERTISING ACTIONS</t>
+        </is>
+      </c>
+      <c r="B80" s="166" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>HikeBike 1</t>
+        </is>
+      </c>
+      <c r="B81" s="174" t="inlineStr">
+        <is>
+          <t>KEEP. 80 vs BB LLC's 81 - one point off the industry best. Redesign cost is not justified; put the money into media inserts and capacity instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Swift Bike ad</t>
+        </is>
+      </c>
+      <c r="B82" s="174" t="inlineStr">
+        <is>
+          <t>REDESIGN around Speed cues. Strip Mountain/Recreation claims (aerodynamic, racing tires, precision brakes, drop bars, lightweight). Target 77 to match Speed of Lite 1 / The Armstrong 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Do NOT add more ads</t>
+        </is>
+      </c>
+      <c r="B83" s="174" t="inlineStr">
+        <is>
+          <t>The leader runs 2 ads for 4 brands; the last-place firm runs 5 for 5. Quality over count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Combined payoff</t>
+        </is>
+      </c>
+      <c r="B84" s="174" t="inlineStr">
+        <is>
+          <t>Swift Bike brand 72-&gt;77 AND ad 70-&gt;77 lifts Marketing Effectiveness from 0.738 to 0.7675 - past BB LLC's 0.765 to become the industry best. Both fixes are cheap relative to capacity.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>